<commit_message>
📊 Actualizar Abono_VU.xlsx — 25-03-2026, 10:00:52 a. m.
</commit_message>
<xml_diff>
--- a/datos/Abono_VU.xlsx
+++ b/datos/Abono_VU.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://funerariaimchile-my.sharepoint.com/personal/anais_gonzalez_funerariaim_cl/Documents/Dashboard_Control Diario de Ventas/Archivos diarios/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A3295E38-76CD-4A26-94B4-2E75EAF02414}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{A6BFC294-D65A-4329-A3C7-0A7FC2987227}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1131" uniqueCount="423">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1209" uniqueCount="444">
   <si>
     <t>EMPRESA</t>
   </si>
@@ -376,6 +376,39 @@
     <t>56250</t>
   </si>
   <si>
+    <t>1015676</t>
+  </si>
+  <si>
+    <t>24/03/2026</t>
+  </si>
+  <si>
+    <t>ARANCIBIA GAMBOA ROBERTO JAIME</t>
+  </si>
+  <si>
+    <t>4137131-5</t>
+  </si>
+  <si>
+    <t>mafil  6132, Pedro Aguirre Cerda, Santiago, Metropolitana  Casa:</t>
+  </si>
+  <si>
+    <t>Pedro Aguirre Cerda</t>
+  </si>
+  <si>
+    <t>936398005 - 91368496</t>
+  </si>
+  <si>
+    <t>rarancibia430@gmail.com</t>
+  </si>
+  <si>
+    <t>59</t>
+  </si>
+  <si>
+    <t>45746</t>
+  </si>
+  <si>
+    <t>05/05/2026</t>
+  </si>
+  <si>
     <t>1015623</t>
   </si>
   <si>
@@ -625,6 +658,36 @@
     <t>22/04/2026</t>
   </si>
   <si>
+    <t>1015684</t>
+  </si>
+  <si>
+    <t>Nayaret Tatiana Puga Marchant</t>
+  </si>
+  <si>
+    <t>GUERRA LEIVA ANA EDELMIRA</t>
+  </si>
+  <si>
+    <t>11399404-3</t>
+  </si>
+  <si>
+    <t>Pampa del tamarugal, ALT 456 - Quilicura -</t>
+  </si>
+  <si>
+    <t>957359715</t>
+  </si>
+  <si>
+    <t>942854716</t>
+  </si>
+  <si>
+    <t>edelmiraguerraleiv@gmail.com - EDELMIRAGUERRALEIV@</t>
+  </si>
+  <si>
+    <t>24</t>
+  </si>
+  <si>
+    <t>24/04/2026</t>
+  </si>
+  <si>
     <t>1015632</t>
   </si>
   <si>
@@ -730,13 +793,10 @@
     <t>Los espinos , ALT 138 - Lampa -</t>
   </si>
   <si>
-    <t>931276144</t>
-  </si>
-  <si>
-    <t>irisvenegas260@gmail.com</t>
-  </si>
-  <si>
-    <t>24</t>
+    <t>931276144 - 56931276144</t>
+  </si>
+  <si>
+    <t>irisvenegas260@gmail.com - IRISVENEGAS260@GMAIL.CO</t>
   </si>
   <si>
     <t>155250</t>
@@ -829,337 +889,343 @@
     <t>99770</t>
   </si>
   <si>
-    <t>1015665</t>
+    <t>1015633</t>
+  </si>
+  <si>
+    <t>VIVIANA HERNANDEZ</t>
+  </si>
+  <si>
+    <t>ALEJANDRA VERDUGO</t>
+  </si>
+  <si>
+    <t>LEYTON CORVALAN BELEN ANDREA</t>
+  </si>
+  <si>
+    <t>21597118-k</t>
+  </si>
+  <si>
+    <t>Pasaje coral de año nuevo, ALT 513 - La Granja -</t>
+  </si>
+  <si>
+    <t>La Granja</t>
+  </si>
+  <si>
+    <t>994206017</t>
+  </si>
+  <si>
+    <t>bleytoncorvalan957@gmail.com</t>
+  </si>
+  <si>
+    <t>Valle De Las Rosas (cuotas)</t>
+  </si>
+  <si>
+    <t>Valle De Las Rosas</t>
+  </si>
+  <si>
+    <t>5880000</t>
+  </si>
+  <si>
+    <t>588000</t>
+  </si>
+  <si>
+    <t>5292000</t>
+  </si>
+  <si>
+    <t>147000</t>
+  </si>
+  <si>
+    <t>1015631</t>
+  </si>
+  <si>
+    <t>NF CARTERA</t>
+  </si>
+  <si>
+    <t>CAYUN HEREDIA KAREN ANDREA</t>
+  </si>
+  <si>
+    <t>18190149-7</t>
+  </si>
+  <si>
+    <t>pasaje  estacion loncoche, ALT 228 - Huechuraba -</t>
+  </si>
+  <si>
+    <t>Huechuraba</t>
+  </si>
+  <si>
+    <t>920512919</t>
+  </si>
+  <si>
+    <t>920234538</t>
+  </si>
+  <si>
+    <t>KARENCAYUNHEREDIA@GMAIL.COM</t>
+  </si>
+  <si>
+    <t>4533000</t>
+  </si>
+  <si>
+    <t>77.09</t>
+  </si>
+  <si>
+    <t>1347000</t>
+  </si>
+  <si>
+    <t>1</t>
+  </si>
+  <si>
+    <t>10/04/2026</t>
+  </si>
+  <si>
+    <t>1015606</t>
+  </si>
+  <si>
+    <t>MADRID GAETE NICXA VIVIANA</t>
+  </si>
+  <si>
+    <t>19586921-9</t>
+  </si>
+  <si>
+    <t>Psje jose carreno trujillo, ALT 1675 - Lampa -</t>
+  </si>
+  <si>
+    <t>935565885</t>
+  </si>
+  <si>
+    <t>nixa@gmail.com</t>
+  </si>
+  <si>
+    <t>59847</t>
+  </si>
+  <si>
+    <t>1015629</t>
+  </si>
+  <si>
+    <t>RODRIGUEZ ESPINOZA ALONSO</t>
+  </si>
+  <si>
+    <t>22318996-2</t>
+  </si>
+  <si>
+    <t>cienfuegos 5455, ALT 5455 - Pedro Aguirre Cerda -</t>
+  </si>
+  <si>
+    <t>978737691</t>
+  </si>
+  <si>
+    <t>alonsorodriguezespinoza1904@gmail.com</t>
+  </si>
+  <si>
+    <t>3990000</t>
+  </si>
+  <si>
+    <t>79.96</t>
+  </si>
+  <si>
+    <t>1000000</t>
+  </si>
+  <si>
+    <t>3</t>
+  </si>
+  <si>
+    <t>3-BA-43</t>
+  </si>
+  <si>
+    <t>Valle de la Memoria</t>
+  </si>
+  <si>
+    <t>1015647</t>
+  </si>
+  <si>
+    <t>ERNESTO OLIVA</t>
+  </si>
+  <si>
+    <t>MIGUEL SANDOVAL</t>
+  </si>
+  <si>
+    <t>ANDREA CONCHA ADASME</t>
+  </si>
+  <si>
+    <t>17/03/2026</t>
+  </si>
+  <si>
+    <t>LLANCALEO ZAMORANO SILVANA VALENTINA</t>
+  </si>
+  <si>
+    <t>15957544-6</t>
+  </si>
+  <si>
+    <t>Av lo cruzat  525, Quilicura, Santiago, Metropolitana  Pi/dp 722 Casa:  Edificio 7</t>
+  </si>
+  <si>
+    <t>994481549</t>
+  </si>
+  <si>
+    <t>Silvll84@gmail.com</t>
+  </si>
+  <si>
+    <t>1300000</t>
+  </si>
+  <si>
+    <t>0.26</t>
+  </si>
+  <si>
+    <t>499000</t>
+  </si>
+  <si>
+    <t>4491000</t>
+  </si>
+  <si>
+    <t>3191000</t>
+  </si>
+  <si>
+    <t>265913</t>
+  </si>
+  <si>
+    <t>4-Z-42</t>
+  </si>
+  <si>
+    <t>Valle de la Memoria 2</t>
+  </si>
+  <si>
+    <t>1015610</t>
+  </si>
+  <si>
+    <t>YIPSY JOSE BRITO MARIN</t>
+  </si>
+  <si>
+    <t>LOPEZ RUIZ SILVIA TERESA</t>
+  </si>
+  <si>
+    <t>10557587-4</t>
+  </si>
+  <si>
+    <t>Juan de Dios marticorena, ALT 6 - Lampa -</t>
+  </si>
+  <si>
+    <t>942671991</t>
+  </si>
+  <si>
+    <t>stlopezr1@gmail.com</t>
+  </si>
+  <si>
+    <t>310500</t>
+  </si>
+  <si>
+    <t>345000</t>
+  </si>
+  <si>
+    <t>3105000</t>
+  </si>
+  <si>
+    <t>2794500</t>
+  </si>
+  <si>
+    <t>46575</t>
+  </si>
+  <si>
+    <t>4</t>
+  </si>
+  <si>
+    <t>04/04/2026</t>
+  </si>
+  <si>
+    <t>7-A-032</t>
+  </si>
+  <si>
+    <t>Valle del Descanso</t>
+  </si>
+  <si>
+    <t>1015609</t>
+  </si>
+  <si>
+    <t>GERENCIA DE VENTAS</t>
+  </si>
+  <si>
+    <t>RODOLFO SANTANA BASAEZ</t>
+  </si>
+  <si>
+    <t>Micaela Tais Vargas Castillo</t>
+  </si>
+  <si>
+    <t>GALAZ ORELLANA YSKRA</t>
+  </si>
+  <si>
+    <t>12859425-6</t>
+  </si>
+  <si>
+    <t>El boldo 8064, Lo Prado, Santiago, Metropolitana  Pi/dp Block 15 Casa:</t>
+  </si>
+  <si>
+    <t>Lo Prado</t>
+  </si>
+  <si>
+    <t>999250322</t>
+  </si>
+  <si>
+    <t>gatubela1@live.cl</t>
+  </si>
+  <si>
+    <t>618000</t>
+  </si>
+  <si>
+    <t>17.91</t>
+  </si>
+  <si>
+    <t>2832000</t>
+  </si>
+  <si>
+    <t>2532000</t>
+  </si>
+  <si>
+    <t>72</t>
+  </si>
+  <si>
+    <t>35143</t>
+  </si>
+  <si>
+    <t>7-A-033</t>
+  </si>
+  <si>
+    <t>1015681</t>
+  </si>
+  <si>
+    <t>IBAÑEZ NUÑEZ CONSTANZA JANICE</t>
+  </si>
+  <si>
+    <t>17680901-9</t>
+  </si>
+  <si>
+    <t>Antonio Maceo 3176, ALT 3176 - Renca -</t>
+  </si>
+  <si>
+    <t>Renca</t>
+  </si>
+  <si>
+    <t>933158189</t>
+  </si>
+  <si>
+    <t>constanzajanice@gmaim.com</t>
   </si>
   <si>
     <t>600000</t>
   </si>
   <si>
-    <t>IBAÑEZ NUÑEZ CONSTANZA JANICE</t>
-  </si>
-  <si>
-    <t>17680901-9</t>
-  </si>
-  <si>
-    <t>Antonio Maceo 3176, ALT 3176 - Renca -</t>
-  </si>
-  <si>
-    <t>Renca</t>
-  </si>
-  <si>
-    <t>933158189</t>
-  </si>
-  <si>
-    <t>constanzajanice@gmaim.com</t>
-  </si>
-  <si>
-    <t>Valle De Las Rosas (cuotas)</t>
-  </si>
-  <si>
-    <t>Valle De Las Rosas</t>
-  </si>
-  <si>
-    <t>5880000</t>
-  </si>
-  <si>
     <t>5280000</t>
   </si>
   <si>
-    <t>146666.66</t>
-  </si>
-  <si>
-    <t>2026-03-13T00:00:00</t>
-  </si>
-  <si>
-    <t>1015633</t>
-  </si>
-  <si>
-    <t>VIVIANA HERNANDEZ</t>
-  </si>
-  <si>
-    <t>ALEJANDRA VERDUGO</t>
-  </si>
-  <si>
-    <t>LEYTON CORVALAN BELEN ANDREA</t>
-  </si>
-  <si>
-    <t>21597118-k</t>
-  </si>
-  <si>
-    <t>Pasaje coral de año nuevo, ALT 513 - La Granja -</t>
-  </si>
-  <si>
-    <t>La Granja</t>
-  </si>
-  <si>
-    <t>994206017</t>
-  </si>
-  <si>
-    <t>bleytoncorvalan957@gmail.com</t>
-  </si>
-  <si>
-    <t>588000</t>
-  </si>
-  <si>
-    <t>5292000</t>
-  </si>
-  <si>
-    <t>147000</t>
-  </si>
-  <si>
-    <t>1015631</t>
-  </si>
-  <si>
-    <t>NF CARTERA</t>
-  </si>
-  <si>
-    <t>CAYUN HEREDIA KAREN ANDREA</t>
-  </si>
-  <si>
-    <t>18190149-7</t>
-  </si>
-  <si>
-    <t>pasaje  estacion loncoche, ALT 228 - Huechuraba -</t>
-  </si>
-  <si>
-    <t>Huechuraba</t>
-  </si>
-  <si>
-    <t>920512919</t>
-  </si>
-  <si>
-    <t>920234538</t>
-  </si>
-  <si>
-    <t>KARENCAYUNHEREDIA@GMAIL.COM</t>
-  </si>
-  <si>
-    <t>4533000</t>
-  </si>
-  <si>
-    <t>77.09</t>
-  </si>
-  <si>
-    <t>1347000</t>
-  </si>
-  <si>
-    <t>1</t>
-  </si>
-  <si>
-    <t>10/04/2026</t>
-  </si>
-  <si>
-    <t>1015606</t>
-  </si>
-  <si>
-    <t>MADRID GAETE NICXA VIVIANA</t>
-  </si>
-  <si>
-    <t>19586921-9</t>
-  </si>
-  <si>
-    <t>Psje jose carreno trujillo, ALT 1675 - Lampa -</t>
-  </si>
-  <si>
-    <t>935565885</t>
-  </si>
-  <si>
-    <t>nixa@gmail.com</t>
-  </si>
-  <si>
-    <t>59847</t>
-  </si>
-  <si>
-    <t>1015629</t>
-  </si>
-  <si>
-    <t>RODRIGUEZ ESPINOZA ALONSO</t>
-  </si>
-  <si>
-    <t>22318996-2</t>
-  </si>
-  <si>
-    <t>cienfuegos 5455, ALT 5455 - Pedro Aguirre Cerda -</t>
-  </si>
-  <si>
-    <t>Pedro Aguirre Cerda</t>
-  </si>
-  <si>
-    <t>978737691</t>
-  </si>
-  <si>
-    <t>alonsorodriguezespinoza1904@gmail.com</t>
-  </si>
-  <si>
-    <t>3990000</t>
-  </si>
-  <si>
-    <t>79.96</t>
-  </si>
-  <si>
-    <t>1000000</t>
-  </si>
-  <si>
-    <t>3</t>
-  </si>
-  <si>
-    <t>3-BA-43</t>
-  </si>
-  <si>
-    <t>Valle de la Memoria</t>
-  </si>
-  <si>
-    <t>1015647</t>
-  </si>
-  <si>
-    <t>ERNESTO OLIVA</t>
-  </si>
-  <si>
-    <t>MIGUEL SANDOVAL</t>
-  </si>
-  <si>
-    <t>ANDREA CONCHA ADASME</t>
-  </si>
-  <si>
-    <t>17/03/2026</t>
-  </si>
-  <si>
-    <t>LLANCALEO ZAMORANO SILVANA VALENTINA</t>
-  </si>
-  <si>
-    <t>15957544-6</t>
-  </si>
-  <si>
-    <t>Av lo cruzat  525, Quilicura, Santiago, Metropolitana  Pi/dp 722 Casa:  Edificio 7</t>
-  </si>
-  <si>
-    <t>994481549</t>
-  </si>
-  <si>
-    <t>Silvll84@gmail.com</t>
-  </si>
-  <si>
-    <t>1300000</t>
-  </si>
-  <si>
-    <t>0.26</t>
-  </si>
-  <si>
-    <t>499000</t>
-  </si>
-  <si>
-    <t>4491000</t>
-  </si>
-  <si>
-    <t>3191000</t>
-  </si>
-  <si>
-    <t>265913</t>
-  </si>
-  <si>
-    <t>4-Z-42</t>
-  </si>
-  <si>
-    <t>Valle de la Memoria 2</t>
-  </si>
-  <si>
-    <t>1015610</t>
-  </si>
-  <si>
-    <t>YIPSY JOSE BRITO MARIN</t>
-  </si>
-  <si>
-    <t>LOPEZ RUIZ SILVIA TERESA</t>
-  </si>
-  <si>
-    <t>10557587-4</t>
-  </si>
-  <si>
-    <t>Juan de Dios marticorena, ALT 6 - Lampa -</t>
-  </si>
-  <si>
-    <t>942671991</t>
-  </si>
-  <si>
-    <t>stlopezr1@gmail.com</t>
-  </si>
-  <si>
-    <t>310500</t>
-  </si>
-  <si>
-    <t>345000</t>
-  </si>
-  <si>
-    <t>3105000</t>
-  </si>
-  <si>
-    <t>2794500</t>
-  </si>
-  <si>
-    <t>46575</t>
-  </si>
-  <si>
-    <t>4</t>
-  </si>
-  <si>
-    <t>04/04/2026</t>
-  </si>
-  <si>
-    <t>7-A-032</t>
-  </si>
-  <si>
-    <t>Valle del Descanso</t>
-  </si>
-  <si>
-    <t>1015609</t>
-  </si>
-  <si>
-    <t>GERENCIA DE VENTAS</t>
-  </si>
-  <si>
-    <t>RODOLFO SANTANA BASAEZ</t>
-  </si>
-  <si>
-    <t>Micaela Tais Vargas Castillo</t>
-  </si>
-  <si>
-    <t>GALAZ ORELLANA YSKRA</t>
-  </si>
-  <si>
-    <t>12859425-6</t>
-  </si>
-  <si>
-    <t>El boldo 8064, Lo Prado, Santiago, Metropolitana  Pi/dp Block 15 Casa:</t>
-  </si>
-  <si>
-    <t>Lo Prado</t>
-  </si>
-  <si>
-    <t>999250322</t>
-  </si>
-  <si>
-    <t>gatubela1@live.cl</t>
-  </si>
-  <si>
-    <t>618000</t>
-  </si>
-  <si>
-    <t>17.91</t>
-  </si>
-  <si>
-    <t>2832000</t>
-  </si>
-  <si>
-    <t>2532000</t>
-  </si>
-  <si>
-    <t>72</t>
-  </si>
-  <si>
-    <t>35143</t>
-  </si>
-  <si>
-    <t>7-A-033</t>
+    <t>146655</t>
+  </si>
+  <si>
+    <t>8</t>
+  </si>
+  <si>
+    <t>08/05/2026</t>
+  </si>
+  <si>
+    <t>1-X-18</t>
+  </si>
+  <si>
+    <t>Valles De las Rosas</t>
   </si>
   <si>
     <t>1015620</t>
@@ -1181,9 +1247,6 @@
   </si>
   <si>
     <t>66553</t>
-  </si>
-  <si>
-    <t>8</t>
   </si>
   <si>
     <t>08/04/2026</t>
@@ -2149,7 +2212,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AM29"/>
+  <dimension ref="A1:AM31"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="39" width="8" customWidth="1"/>
@@ -2877,10 +2940,10 @@
         <v>118</v>
       </c>
       <c r="C7" t="s">
-        <v>119</v>
+        <v>41</v>
       </c>
       <c r="D7" t="s">
-        <v>120</v>
+        <v>42</v>
       </c>
       <c r="E7" t="s">
         <v>43</v>
@@ -2889,22 +2952,22 @@
         <v>44</v>
       </c>
       <c r="G7" t="s">
-        <v>45</v>
+        <v>77</v>
       </c>
       <c r="H7" t="s">
-        <v>46</v>
+        <v>78</v>
       </c>
       <c r="I7" t="s">
-        <v>44</v>
+        <v>119</v>
       </c>
       <c r="J7" t="s">
+        <v>120</v>
+      </c>
+      <c r="K7" t="s">
         <v>121</v>
       </c>
-      <c r="K7" t="s">
+      <c r="L7" t="s">
         <v>122</v>
-      </c>
-      <c r="L7" t="s">
-        <v>123</v>
       </c>
       <c r="M7" t="s">
         <v>51</v>
@@ -2913,7 +2976,7 @@
         <v>52</v>
       </c>
       <c r="O7" t="s">
-        <v>53</v>
+        <v>123</v>
       </c>
       <c r="P7" t="s">
         <v>44</v>
@@ -2955,7 +3018,7 @@
         <v>58</v>
       </c>
       <c r="AC7" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="AD7" t="s">
         <v>62</v>
@@ -2964,16 +3027,16 @@
         <v>63</v>
       </c>
       <c r="AF7" t="s">
-        <v>64</v>
+        <v>126</v>
       </c>
       <c r="AG7" t="s">
-        <v>65</v>
+        <v>127</v>
       </c>
       <c r="AH7" t="s">
-        <v>126</v>
+        <v>104</v>
       </c>
       <c r="AI7" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="AJ7" t="s">
         <v>44</v>
@@ -2985,7 +3048,7 @@
         <v>44</v>
       </c>
       <c r="AM7" t="s">
-        <v>128</v>
+        <v>44</v>
       </c>
     </row>
     <row r="8" spans="1:39" x14ac:dyDescent="0.3">
@@ -2996,10 +3059,10 @@
         <v>129</v>
       </c>
       <c r="C8" t="s">
-        <v>41</v>
+        <v>130</v>
       </c>
       <c r="D8" t="s">
-        <v>42</v>
+        <v>131</v>
       </c>
       <c r="E8" t="s">
         <v>43</v>
@@ -3014,16 +3077,16 @@
         <v>46</v>
       </c>
       <c r="I8" t="s">
-        <v>130</v>
+        <v>44</v>
       </c>
       <c r="J8" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="K8" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="L8" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="M8" t="s">
         <v>51</v>
@@ -3038,10 +3101,10 @@
         <v>44</v>
       </c>
       <c r="Q8" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="R8" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="S8" t="s">
         <v>44</v>
@@ -3074,7 +3137,7 @@
         <v>58</v>
       </c>
       <c r="AC8" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="AD8" t="s">
         <v>62</v>
@@ -3083,16 +3146,16 @@
         <v>63</v>
       </c>
       <c r="AF8" t="s">
-        <v>93</v>
+        <v>64</v>
       </c>
       <c r="AG8" t="s">
-        <v>117</v>
+        <v>65</v>
       </c>
       <c r="AH8" t="s">
-        <v>89</v>
+        <v>137</v>
       </c>
       <c r="AI8" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="AJ8" t="s">
         <v>44</v>
@@ -3104,7 +3167,7 @@
         <v>44</v>
       </c>
       <c r="AM8" t="s">
-        <v>44</v>
+        <v>139</v>
       </c>
     </row>
     <row r="9" spans="1:39" x14ac:dyDescent="0.3">
@@ -3112,13 +3175,13 @@
         <v>39</v>
       </c>
       <c r="B9" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="C9" t="s">
         <v>41</v>
       </c>
       <c r="D9" t="s">
-        <v>138</v>
+        <v>42</v>
       </c>
       <c r="E9" t="s">
         <v>43</v>
@@ -3127,22 +3190,22 @@
         <v>44</v>
       </c>
       <c r="G9" t="s">
-        <v>69</v>
+        <v>45</v>
       </c>
       <c r="H9" t="s">
-        <v>139</v>
+        <v>46</v>
       </c>
       <c r="I9" t="s">
-        <v>130</v>
+        <v>141</v>
       </c>
       <c r="J9" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="K9" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="L9" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="M9" t="s">
         <v>51</v>
@@ -3154,13 +3217,13 @@
         <v>53</v>
       </c>
       <c r="P9" t="s">
-        <v>143</v>
+        <v>44</v>
       </c>
       <c r="Q9" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="R9" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="S9" t="s">
         <v>44</v>
@@ -3202,16 +3265,16 @@
         <v>63</v>
       </c>
       <c r="AF9" t="s">
-        <v>64</v>
+        <v>93</v>
       </c>
       <c r="AG9" t="s">
-        <v>65</v>
+        <v>117</v>
       </c>
       <c r="AH9" t="s">
         <v>89</v>
       </c>
       <c r="AI9" t="s">
-        <v>136</v>
+        <v>147</v>
       </c>
       <c r="AJ9" t="s">
         <v>44</v>
@@ -3223,7 +3286,7 @@
         <v>44</v>
       </c>
       <c r="AM9" t="s">
-        <v>146</v>
+        <v>44</v>
       </c>
     </row>
     <row r="10" spans="1:39" x14ac:dyDescent="0.3">
@@ -3231,13 +3294,13 @@
         <v>39</v>
       </c>
       <c r="B10" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="C10" t="s">
         <v>41</v>
       </c>
       <c r="D10" t="s">
-        <v>42</v>
+        <v>149</v>
       </c>
       <c r="E10" t="s">
         <v>43</v>
@@ -3246,22 +3309,22 @@
         <v>44</v>
       </c>
       <c r="G10" t="s">
-        <v>45</v>
+        <v>69</v>
       </c>
       <c r="H10" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="I10" t="s">
-        <v>130</v>
+        <v>141</v>
       </c>
       <c r="J10" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="K10" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="L10" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="M10" t="s">
         <v>51</v>
@@ -3273,64 +3336,64 @@
         <v>53</v>
       </c>
       <c r="P10" t="s">
-        <v>44</v>
+        <v>154</v>
       </c>
       <c r="Q10" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="R10" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="S10" t="s">
         <v>44</v>
       </c>
       <c r="T10" t="s">
-        <v>154</v>
+        <v>56</v>
       </c>
       <c r="U10" t="s">
-        <v>154</v>
+        <v>56</v>
       </c>
       <c r="V10" t="s">
         <v>57</v>
       </c>
       <c r="W10" t="s">
-        <v>155</v>
+        <v>58</v>
       </c>
       <c r="X10" t="s">
-        <v>156</v>
+        <v>59</v>
       </c>
       <c r="Y10" t="s">
-        <v>157</v>
+        <v>60</v>
       </c>
       <c r="Z10" t="s">
-        <v>158</v>
+        <v>42</v>
       </c>
       <c r="AA10" t="s">
-        <v>89</v>
+        <v>42</v>
       </c>
       <c r="AB10" t="s">
-        <v>159</v>
+        <v>58</v>
       </c>
       <c r="AC10" t="s">
-        <v>160</v>
+        <v>61</v>
       </c>
       <c r="AD10" t="s">
-        <v>161</v>
+        <v>62</v>
       </c>
       <c r="AE10" t="s">
         <v>63</v>
       </c>
       <c r="AF10" t="s">
-        <v>162</v>
+        <v>64</v>
       </c>
       <c r="AG10" t="s">
-        <v>163</v>
+        <v>65</v>
       </c>
       <c r="AH10" t="s">
         <v>89</v>
       </c>
       <c r="AI10" t="s">
-        <v>136</v>
+        <v>147</v>
       </c>
       <c r="AJ10" t="s">
         <v>44</v>
@@ -3342,7 +3405,7 @@
         <v>44</v>
       </c>
       <c r="AM10" t="s">
-        <v>44</v>
+        <v>157</v>
       </c>
     </row>
     <row r="11" spans="1:39" x14ac:dyDescent="0.3">
@@ -3350,7 +3413,7 @@
         <v>39</v>
       </c>
       <c r="B11" t="s">
-        <v>164</v>
+        <v>158</v>
       </c>
       <c r="C11" t="s">
         <v>41</v>
@@ -3365,91 +3428,91 @@
         <v>44</v>
       </c>
       <c r="G11" t="s">
-        <v>69</v>
+        <v>45</v>
       </c>
       <c r="H11" t="s">
-        <v>107</v>
+        <v>159</v>
       </c>
       <c r="I11" t="s">
+        <v>141</v>
+      </c>
+      <c r="J11" t="s">
+        <v>160</v>
+      </c>
+      <c r="K11" t="s">
+        <v>161</v>
+      </c>
+      <c r="L11" t="s">
+        <v>162</v>
+      </c>
+      <c r="M11" t="s">
+        <v>51</v>
+      </c>
+      <c r="N11" t="s">
+        <v>52</v>
+      </c>
+      <c r="O11" t="s">
+        <v>53</v>
+      </c>
+      <c r="P11" t="s">
+        <v>44</v>
+      </c>
+      <c r="Q11" t="s">
+        <v>163</v>
+      </c>
+      <c r="R11" t="s">
+        <v>164</v>
+      </c>
+      <c r="S11" t="s">
+        <v>44</v>
+      </c>
+      <c r="T11" t="s">
         <v>165</v>
       </c>
-      <c r="J11" t="s">
-        <v>166</v>
-      </c>
-      <c r="K11" t="s">
-        <v>167</v>
-      </c>
-      <c r="L11" t="s">
-        <v>44</v>
-      </c>
-      <c r="M11" t="s">
-        <v>112</v>
-      </c>
-      <c r="N11" t="s">
-        <v>168</v>
-      </c>
-      <c r="O11" t="s">
-        <v>44</v>
-      </c>
-      <c r="P11" t="s">
-        <v>169</v>
-      </c>
-      <c r="Q11" t="s">
-        <v>169</v>
-      </c>
-      <c r="R11" t="s">
-        <v>170</v>
-      </c>
-      <c r="S11" t="s">
-        <v>44</v>
-      </c>
-      <c r="T11" t="s">
-        <v>154</v>
-      </c>
       <c r="U11" t="s">
-        <v>154</v>
+        <v>165</v>
       </c>
       <c r="V11" t="s">
         <v>57</v>
       </c>
       <c r="W11" t="s">
-        <v>155</v>
+        <v>166</v>
       </c>
       <c r="X11" t="s">
+        <v>167</v>
+      </c>
+      <c r="Y11" t="s">
+        <v>168</v>
+      </c>
+      <c r="Z11" t="s">
+        <v>169</v>
+      </c>
+      <c r="AA11" t="s">
+        <v>89</v>
+      </c>
+      <c r="AB11" t="s">
+        <v>170</v>
+      </c>
+      <c r="AC11" t="s">
         <v>171</v>
       </c>
-      <c r="Y11" t="s">
-        <v>87</v>
-      </c>
-      <c r="Z11" t="s">
+      <c r="AD11" t="s">
         <v>172</v>
-      </c>
-      <c r="AA11" t="s">
-        <v>173</v>
-      </c>
-      <c r="AB11" t="s">
-        <v>174</v>
-      </c>
-      <c r="AC11" t="s">
-        <v>175</v>
-      </c>
-      <c r="AD11" t="s">
-        <v>176</v>
       </c>
       <c r="AE11" t="s">
         <v>63</v>
       </c>
       <c r="AF11" t="s">
-        <v>93</v>
+        <v>173</v>
       </c>
       <c r="AG11" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="AH11" t="s">
-        <v>178</v>
+        <v>89</v>
       </c>
       <c r="AI11" t="s">
-        <v>179</v>
+        <v>147</v>
       </c>
       <c r="AJ11" t="s">
         <v>44</v>
@@ -3469,7 +3532,7 @@
         <v>39</v>
       </c>
       <c r="B12" t="s">
-        <v>180</v>
+        <v>175</v>
       </c>
       <c r="C12" t="s">
         <v>41</v>
@@ -3487,88 +3550,88 @@
         <v>69</v>
       </c>
       <c r="H12" t="s">
-        <v>70</v>
+        <v>107</v>
       </c>
       <c r="I12" t="s">
+        <v>176</v>
+      </c>
+      <c r="J12" t="s">
+        <v>177</v>
+      </c>
+      <c r="K12" t="s">
+        <v>178</v>
+      </c>
+      <c r="L12" t="s">
+        <v>44</v>
+      </c>
+      <c r="M12" t="s">
+        <v>112</v>
+      </c>
+      <c r="N12" t="s">
+        <v>179</v>
+      </c>
+      <c r="O12" t="s">
+        <v>44</v>
+      </c>
+      <c r="P12" t="s">
+        <v>180</v>
+      </c>
+      <c r="Q12" t="s">
+        <v>180</v>
+      </c>
+      <c r="R12" t="s">
+        <v>181</v>
+      </c>
+      <c r="S12" t="s">
+        <v>44</v>
+      </c>
+      <c r="T12" t="s">
         <v>165</v>
       </c>
-      <c r="J12" t="s">
-        <v>181</v>
-      </c>
-      <c r="K12" t="s">
-        <v>182</v>
-      </c>
-      <c r="L12" t="s">
-        <v>183</v>
-      </c>
-      <c r="M12" t="s">
-        <v>51</v>
-      </c>
-      <c r="N12" t="s">
-        <v>184</v>
-      </c>
-      <c r="O12" t="s">
-        <v>185</v>
-      </c>
-      <c r="P12" t="s">
-        <v>186</v>
-      </c>
-      <c r="Q12" t="s">
-        <v>186</v>
-      </c>
-      <c r="R12" t="s">
-        <v>187</v>
-      </c>
-      <c r="S12" t="s">
-        <v>44</v>
-      </c>
-      <c r="T12" t="s">
-        <v>56</v>
-      </c>
       <c r="U12" t="s">
-        <v>56</v>
+        <v>165</v>
       </c>
       <c r="V12" t="s">
         <v>57</v>
       </c>
       <c r="W12" t="s">
-        <v>58</v>
+        <v>166</v>
       </c>
       <c r="X12" t="s">
-        <v>59</v>
+        <v>182</v>
       </c>
       <c r="Y12" t="s">
-        <v>60</v>
+        <v>87</v>
       </c>
       <c r="Z12" t="s">
-        <v>42</v>
+        <v>183</v>
       </c>
       <c r="AA12" t="s">
-        <v>42</v>
+        <v>184</v>
       </c>
       <c r="AB12" t="s">
-        <v>58</v>
+        <v>185</v>
       </c>
       <c r="AC12" t="s">
-        <v>61</v>
+        <v>186</v>
       </c>
       <c r="AD12" t="s">
-        <v>62</v>
+        <v>187</v>
       </c>
       <c r="AE12" t="s">
         <v>63</v>
       </c>
       <c r="AF12" t="s">
+        <v>93</v>
+      </c>
+      <c r="AG12" t="s">
         <v>188</v>
       </c>
-      <c r="AG12" t="s">
+      <c r="AH12" t="s">
         <v>189</v>
       </c>
-      <c r="AH12" t="s">
-        <v>178</v>
-      </c>
       <c r="AI12" t="s">
-        <v>179</v>
+        <v>190</v>
       </c>
       <c r="AJ12" t="s">
         <v>44</v>
@@ -3588,7 +3651,7 @@
         <v>39</v>
       </c>
       <c r="B13" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="C13" t="s">
         <v>41</v>
@@ -3603,13 +3666,13 @@
         <v>44</v>
       </c>
       <c r="G13" t="s">
-        <v>77</v>
+        <v>69</v>
       </c>
       <c r="H13" t="s">
-        <v>191</v>
+        <v>70</v>
       </c>
       <c r="I13" t="s">
-        <v>165</v>
+        <v>176</v>
       </c>
       <c r="J13" t="s">
         <v>192</v>
@@ -3624,70 +3687,70 @@
         <v>51</v>
       </c>
       <c r="N13" t="s">
-        <v>52</v>
+        <v>195</v>
       </c>
       <c r="O13" t="s">
-        <v>53</v>
+        <v>196</v>
       </c>
       <c r="P13" t="s">
-        <v>44</v>
+        <v>197</v>
       </c>
       <c r="Q13" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="R13" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="S13" t="s">
         <v>44</v>
       </c>
       <c r="T13" t="s">
-        <v>154</v>
+        <v>56</v>
       </c>
       <c r="U13" t="s">
-        <v>154</v>
+        <v>56</v>
       </c>
       <c r="V13" t="s">
         <v>57</v>
       </c>
       <c r="W13" t="s">
-        <v>155</v>
+        <v>58</v>
       </c>
       <c r="X13" t="s">
-        <v>172</v>
+        <v>59</v>
       </c>
       <c r="Y13" t="s">
         <v>60</v>
       </c>
       <c r="Z13" t="s">
-        <v>172</v>
+        <v>42</v>
       </c>
       <c r="AA13" t="s">
-        <v>173</v>
+        <v>42</v>
       </c>
       <c r="AB13" t="s">
-        <v>174</v>
+        <v>58</v>
       </c>
       <c r="AC13" t="s">
-        <v>175</v>
+        <v>61</v>
       </c>
       <c r="AD13" t="s">
-        <v>197</v>
+        <v>62</v>
       </c>
       <c r="AE13" t="s">
         <v>63</v>
       </c>
       <c r="AF13" t="s">
-        <v>93</v>
+        <v>199</v>
       </c>
       <c r="AG13" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="AH13" t="s">
-        <v>199</v>
+        <v>189</v>
       </c>
       <c r="AI13" t="s">
-        <v>200</v>
+        <v>190</v>
       </c>
       <c r="AJ13" t="s">
         <v>44</v>
@@ -3722,22 +3785,22 @@
         <v>44</v>
       </c>
       <c r="G14" t="s">
-        <v>69</v>
+        <v>77</v>
       </c>
       <c r="H14" t="s">
         <v>202</v>
       </c>
       <c r="I14" t="s">
+        <v>176</v>
+      </c>
+      <c r="J14" t="s">
         <v>203</v>
       </c>
-      <c r="J14" t="s">
+      <c r="K14" t="s">
         <v>204</v>
       </c>
-      <c r="K14" t="s">
+      <c r="L14" t="s">
         <v>205</v>
-      </c>
-      <c r="L14" t="s">
-        <v>206</v>
       </c>
       <c r="M14" t="s">
         <v>51</v>
@@ -3749,58 +3812,58 @@
         <v>53</v>
       </c>
       <c r="P14" t="s">
+        <v>44</v>
+      </c>
+      <c r="Q14" t="s">
+        <v>206</v>
+      </c>
+      <c r="R14" t="s">
         <v>207</v>
       </c>
-      <c r="Q14" t="s">
-        <v>208</v>
-      </c>
-      <c r="R14" t="s">
-        <v>209</v>
-      </c>
       <c r="S14" t="s">
         <v>44</v>
       </c>
       <c r="T14" t="s">
-        <v>56</v>
+        <v>165</v>
       </c>
       <c r="U14" t="s">
-        <v>56</v>
+        <v>165</v>
       </c>
       <c r="V14" t="s">
         <v>57</v>
       </c>
       <c r="W14" t="s">
-        <v>58</v>
+        <v>166</v>
       </c>
       <c r="X14" t="s">
-        <v>59</v>
+        <v>183</v>
       </c>
       <c r="Y14" t="s">
         <v>60</v>
       </c>
       <c r="Z14" t="s">
-        <v>42</v>
+        <v>183</v>
       </c>
       <c r="AA14" t="s">
-        <v>42</v>
+        <v>184</v>
       </c>
       <c r="AB14" t="s">
-        <v>58</v>
+        <v>185</v>
       </c>
       <c r="AC14" t="s">
-        <v>61</v>
+        <v>186</v>
       </c>
       <c r="AD14" t="s">
-        <v>62</v>
+        <v>208</v>
       </c>
       <c r="AE14" t="s">
         <v>63</v>
       </c>
       <c r="AF14" t="s">
-        <v>64</v>
+        <v>93</v>
       </c>
       <c r="AG14" t="s">
-        <v>65</v>
+        <v>209</v>
       </c>
       <c r="AH14" t="s">
         <v>210</v>
@@ -3832,7 +3895,7 @@
         <v>41</v>
       </c>
       <c r="D15" t="s">
-        <v>213</v>
+        <v>42</v>
       </c>
       <c r="E15" t="s">
         <v>43</v>
@@ -3841,22 +3904,22 @@
         <v>44</v>
       </c>
       <c r="G15" t="s">
-        <v>45</v>
+        <v>77</v>
       </c>
       <c r="H15" t="s">
+        <v>213</v>
+      </c>
+      <c r="I15" t="s">
+        <v>119</v>
+      </c>
+      <c r="J15" t="s">
         <v>214</v>
       </c>
-      <c r="I15" t="s">
-        <v>47</v>
-      </c>
-      <c r="J15" t="s">
+      <c r="K15" t="s">
         <v>215</v>
       </c>
-      <c r="K15" t="s">
+      <c r="L15" t="s">
         <v>216</v>
-      </c>
-      <c r="L15" t="s">
-        <v>217</v>
       </c>
       <c r="M15" t="s">
         <v>51</v>
@@ -3868,7 +3931,7 @@
         <v>53</v>
       </c>
       <c r="P15" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="Q15" t="s">
         <v>218</v>
@@ -3880,52 +3943,52 @@
         <v>44</v>
       </c>
       <c r="T15" t="s">
-        <v>84</v>
+        <v>56</v>
       </c>
       <c r="U15" t="s">
-        <v>84</v>
+        <v>56</v>
       </c>
       <c r="V15" t="s">
         <v>57</v>
       </c>
       <c r="W15" t="s">
-        <v>85</v>
+        <v>58</v>
       </c>
       <c r="X15" t="s">
-        <v>220</v>
+        <v>59</v>
       </c>
       <c r="Y15" t="s">
         <v>60</v>
       </c>
       <c r="Z15" t="s">
-        <v>221</v>
+        <v>42</v>
       </c>
       <c r="AA15" t="s">
-        <v>222</v>
+        <v>42</v>
       </c>
       <c r="AB15" t="s">
-        <v>223</v>
+        <v>58</v>
       </c>
       <c r="AC15" t="s">
-        <v>224</v>
+        <v>61</v>
       </c>
       <c r="AD15" t="s">
-        <v>225</v>
+        <v>62</v>
       </c>
       <c r="AE15" t="s">
         <v>63</v>
       </c>
       <c r="AF15" t="s">
-        <v>64</v>
+        <v>126</v>
       </c>
       <c r="AG15" t="s">
-        <v>226</v>
+        <v>127</v>
       </c>
       <c r="AH15" t="s">
-        <v>227</v>
+        <v>220</v>
       </c>
       <c r="AI15" t="s">
-        <v>228</v>
+        <v>221</v>
       </c>
       <c r="AJ15" t="s">
         <v>44</v>
@@ -3937,7 +4000,7 @@
         <v>44</v>
       </c>
       <c r="AM15" t="s">
-        <v>229</v>
+        <v>44</v>
       </c>
     </row>
     <row r="16" spans="1:39" x14ac:dyDescent="0.3">
@@ -3945,13 +4008,13 @@
         <v>39</v>
       </c>
       <c r="B16" t="s">
-        <v>230</v>
+        <v>222</v>
       </c>
       <c r="C16" t="s">
-        <v>119</v>
+        <v>41</v>
       </c>
       <c r="D16" t="s">
-        <v>231</v>
+        <v>42</v>
       </c>
       <c r="E16" t="s">
         <v>43</v>
@@ -3963,88 +4026,88 @@
         <v>69</v>
       </c>
       <c r="H16" t="s">
-        <v>232</v>
+        <v>223</v>
       </c>
       <c r="I16" t="s">
-        <v>44</v>
+        <v>224</v>
       </c>
       <c r="J16" t="s">
-        <v>233</v>
+        <v>225</v>
       </c>
       <c r="K16" t="s">
-        <v>234</v>
+        <v>226</v>
       </c>
       <c r="L16" t="s">
-        <v>235</v>
+        <v>227</v>
       </c>
       <c r="M16" t="s">
         <v>51</v>
       </c>
       <c r="N16" t="s">
-        <v>184</v>
+        <v>52</v>
       </c>
       <c r="O16" t="s">
-        <v>185</v>
+        <v>53</v>
       </c>
       <c r="P16" t="s">
-        <v>44</v>
+        <v>228</v>
       </c>
       <c r="Q16" t="s">
-        <v>236</v>
+        <v>229</v>
       </c>
       <c r="R16" t="s">
-        <v>237</v>
+        <v>230</v>
       </c>
       <c r="S16" t="s">
         <v>44</v>
       </c>
       <c r="T16" t="s">
-        <v>154</v>
+        <v>56</v>
       </c>
       <c r="U16" t="s">
-        <v>154</v>
+        <v>56</v>
       </c>
       <c r="V16" t="s">
         <v>57</v>
       </c>
       <c r="W16" t="s">
-        <v>155</v>
+        <v>58</v>
       </c>
       <c r="X16" t="s">
-        <v>171</v>
+        <v>59</v>
       </c>
       <c r="Y16" t="s">
-        <v>87</v>
+        <v>60</v>
       </c>
       <c r="Z16" t="s">
-        <v>172</v>
+        <v>42</v>
       </c>
       <c r="AA16" t="s">
-        <v>173</v>
+        <v>42</v>
       </c>
       <c r="AB16" t="s">
-        <v>174</v>
+        <v>58</v>
       </c>
       <c r="AC16" t="s">
-        <v>174</v>
+        <v>61</v>
       </c>
       <c r="AD16" t="s">
-        <v>176</v>
+        <v>62</v>
       </c>
       <c r="AE16" t="s">
-        <v>44</v>
+        <v>63</v>
       </c>
       <c r="AF16" t="s">
-        <v>238</v>
+        <v>64</v>
       </c>
       <c r="AG16" t="s">
-        <v>239</v>
+        <v>65</v>
       </c>
       <c r="AH16" t="s">
-        <v>240</v>
+        <v>231</v>
       </c>
       <c r="AI16" t="s">
-        <v>241</v>
+        <v>232</v>
       </c>
       <c r="AJ16" t="s">
         <v>44</v>
@@ -4056,7 +4119,7 @@
         <v>44</v>
       </c>
       <c r="AM16" t="s">
-        <v>242</v>
+        <v>44</v>
       </c>
     </row>
     <row r="17" spans="1:39" x14ac:dyDescent="0.3">
@@ -4064,13 +4127,13 @@
         <v>39</v>
       </c>
       <c r="B17" t="s">
-        <v>243</v>
+        <v>233</v>
       </c>
       <c r="C17" t="s">
         <v>41</v>
       </c>
       <c r="D17" t="s">
-        <v>42</v>
+        <v>234</v>
       </c>
       <c r="E17" t="s">
         <v>43</v>
@@ -4079,22 +4142,22 @@
         <v>44</v>
       </c>
       <c r="G17" t="s">
-        <v>69</v>
+        <v>45</v>
       </c>
       <c r="H17" t="s">
-        <v>70</v>
+        <v>235</v>
       </c>
       <c r="I17" t="s">
         <v>47</v>
       </c>
       <c r="J17" t="s">
-        <v>71</v>
+        <v>236</v>
       </c>
       <c r="K17" t="s">
-        <v>72</v>
+        <v>237</v>
       </c>
       <c r="L17" t="s">
-        <v>73</v>
+        <v>238</v>
       </c>
       <c r="M17" t="s">
         <v>51</v>
@@ -4106,49 +4169,49 @@
         <v>53</v>
       </c>
       <c r="P17" t="s">
-        <v>74</v>
+        <v>239</v>
       </c>
       <c r="Q17" t="s">
-        <v>74</v>
+        <v>239</v>
       </c>
       <c r="R17" t="s">
-        <v>75</v>
+        <v>240</v>
       </c>
       <c r="S17" t="s">
-        <v>244</v>
+        <v>44</v>
       </c>
       <c r="T17" t="s">
-        <v>245</v>
+        <v>84</v>
       </c>
       <c r="U17" t="s">
-        <v>246</v>
+        <v>84</v>
       </c>
       <c r="V17" t="s">
         <v>57</v>
       </c>
       <c r="W17" t="s">
-        <v>247</v>
+        <v>85</v>
       </c>
       <c r="X17" t="s">
-        <v>248</v>
+        <v>241</v>
       </c>
       <c r="Y17" t="s">
-        <v>249</v>
+        <v>60</v>
       </c>
       <c r="Z17" t="s">
-        <v>42</v>
+        <v>242</v>
       </c>
       <c r="AA17" t="s">
-        <v>42</v>
+        <v>243</v>
       </c>
       <c r="AB17" t="s">
-        <v>247</v>
+        <v>244</v>
       </c>
       <c r="AC17" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
       <c r="AD17" t="s">
-        <v>250</v>
+        <v>246</v>
       </c>
       <c r="AE17" t="s">
         <v>63</v>
@@ -4157,25 +4220,25 @@
         <v>64</v>
       </c>
       <c r="AG17" t="s">
-        <v>251</v>
+        <v>247</v>
       </c>
       <c r="AH17" t="s">
-        <v>66</v>
+        <v>248</v>
       </c>
       <c r="AI17" t="s">
-        <v>67</v>
+        <v>249</v>
       </c>
       <c r="AJ17" t="s">
         <v>44</v>
       </c>
       <c r="AK17" t="s">
-        <v>252</v>
+        <v>44</v>
       </c>
       <c r="AL17" t="s">
-        <v>253</v>
+        <v>44</v>
       </c>
       <c r="AM17" t="s">
-        <v>44</v>
+        <v>250</v>
       </c>
     </row>
     <row r="18" spans="1:39" x14ac:dyDescent="0.3">
@@ -4183,13 +4246,13 @@
         <v>39</v>
       </c>
       <c r="B18" t="s">
-        <v>254</v>
+        <v>251</v>
       </c>
       <c r="C18" t="s">
-        <v>41</v>
+        <v>130</v>
       </c>
       <c r="D18" t="s">
-        <v>42</v>
+        <v>252</v>
       </c>
       <c r="E18" t="s">
         <v>43</v>
@@ -4201,100 +4264,100 @@
         <v>69</v>
       </c>
       <c r="H18" t="s">
+        <v>253</v>
+      </c>
+      <c r="I18" t="s">
+        <v>44</v>
+      </c>
+      <c r="J18" t="s">
+        <v>254</v>
+      </c>
+      <c r="K18" t="s">
         <v>255</v>
       </c>
-      <c r="I18" t="s">
-        <v>47</v>
-      </c>
-      <c r="J18" t="s">
+      <c r="L18" t="s">
         <v>256</v>
-      </c>
-      <c r="K18" t="s">
-        <v>257</v>
-      </c>
-      <c r="L18" t="s">
-        <v>258</v>
       </c>
       <c r="M18" t="s">
         <v>51</v>
       </c>
       <c r="N18" t="s">
-        <v>52</v>
+        <v>195</v>
       </c>
       <c r="O18" t="s">
-        <v>53</v>
+        <v>196</v>
       </c>
       <c r="P18" t="s">
-        <v>259</v>
+        <v>44</v>
       </c>
       <c r="Q18" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="R18" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="S18" t="s">
-        <v>244</v>
+        <v>44</v>
       </c>
       <c r="T18" t="s">
-        <v>261</v>
+        <v>165</v>
       </c>
       <c r="U18" t="s">
-        <v>262</v>
+        <v>165</v>
       </c>
       <c r="V18" t="s">
         <v>57</v>
       </c>
       <c r="W18" t="s">
-        <v>263</v>
+        <v>166</v>
       </c>
       <c r="X18" t="s">
-        <v>248</v>
+        <v>182</v>
       </c>
       <c r="Y18" t="s">
-        <v>264</v>
+        <v>87</v>
       </c>
       <c r="Z18" t="s">
-        <v>265</v>
+        <v>183</v>
       </c>
       <c r="AA18" t="s">
-        <v>178</v>
+        <v>184</v>
       </c>
       <c r="AB18" t="s">
-        <v>266</v>
+        <v>185</v>
       </c>
       <c r="AC18" t="s">
-        <v>266</v>
+        <v>185</v>
       </c>
       <c r="AD18" t="s">
-        <v>267</v>
+        <v>187</v>
       </c>
       <c r="AE18" t="s">
-        <v>63</v>
+        <v>44</v>
       </c>
       <c r="AF18" t="s">
-        <v>64</v>
+        <v>220</v>
       </c>
       <c r="AG18" t="s">
-        <v>268</v>
+        <v>259</v>
       </c>
       <c r="AH18" t="s">
-        <v>66</v>
+        <v>260</v>
       </c>
       <c r="AI18" t="s">
-        <v>67</v>
+        <v>261</v>
       </c>
       <c r="AJ18" t="s">
         <v>44</v>
       </c>
       <c r="AK18" t="s">
-        <v>252</v>
+        <v>44</v>
       </c>
       <c r="AL18" t="s">
-        <v>253</v>
+        <v>44</v>
       </c>
       <c r="AM18" t="s">
-        <v>44</v>
+        <v>262</v>
       </c>
     </row>
     <row r="19" spans="1:39" x14ac:dyDescent="0.3">
@@ -4302,13 +4365,13 @@
         <v>39</v>
       </c>
       <c r="B19" t="s">
-        <v>269</v>
+        <v>263</v>
       </c>
       <c r="C19" t="s">
         <v>41</v>
       </c>
       <c r="D19" t="s">
-        <v>270</v>
+        <v>42</v>
       </c>
       <c r="E19" t="s">
         <v>43</v>
@@ -4317,22 +4380,22 @@
         <v>44</v>
       </c>
       <c r="G19" t="s">
-        <v>45</v>
+        <v>69</v>
       </c>
       <c r="H19" t="s">
-        <v>46</v>
+        <v>70</v>
       </c>
       <c r="I19" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="J19" t="s">
-        <v>271</v>
+        <v>71</v>
       </c>
       <c r="K19" t="s">
-        <v>272</v>
+        <v>72</v>
       </c>
       <c r="L19" t="s">
-        <v>273</v>
+        <v>73</v>
       </c>
       <c r="M19" t="s">
         <v>51</v>
@@ -4341,37 +4404,37 @@
         <v>52</v>
       </c>
       <c r="O19" t="s">
-        <v>274</v>
+        <v>53</v>
       </c>
       <c r="P19" t="s">
-        <v>44</v>
+        <v>74</v>
       </c>
       <c r="Q19" t="s">
-        <v>275</v>
+        <v>74</v>
       </c>
       <c r="R19" t="s">
-        <v>276</v>
+        <v>75</v>
       </c>
       <c r="S19" t="s">
-        <v>244</v>
+        <v>264</v>
       </c>
       <c r="T19" t="s">
-        <v>277</v>
+        <v>265</v>
       </c>
       <c r="U19" t="s">
-        <v>278</v>
+        <v>266</v>
       </c>
       <c r="V19" t="s">
         <v>57</v>
       </c>
       <c r="W19" t="s">
-        <v>279</v>
+        <v>267</v>
       </c>
       <c r="X19" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="Y19" t="s">
-        <v>60</v>
+        <v>269</v>
       </c>
       <c r="Z19" t="s">
         <v>42</v>
@@ -4380,13 +4443,13 @@
         <v>42</v>
       </c>
       <c r="AB19" t="s">
-        <v>279</v>
+        <v>267</v>
       </c>
       <c r="AC19" t="s">
-        <v>279</v>
+        <v>267</v>
       </c>
       <c r="AD19" t="s">
-        <v>280</v>
+        <v>270</v>
       </c>
       <c r="AE19" t="s">
         <v>63</v>
@@ -4395,7 +4458,7 @@
         <v>64</v>
       </c>
       <c r="AG19" t="s">
-        <v>281</v>
+        <v>271</v>
       </c>
       <c r="AH19" t="s">
         <v>66</v>
@@ -4407,13 +4470,13 @@
         <v>44</v>
       </c>
       <c r="AK19" t="s">
-        <v>252</v>
+        <v>272</v>
       </c>
       <c r="AL19" t="s">
-        <v>253</v>
+        <v>273</v>
       </c>
       <c r="AM19" t="s">
-        <v>282</v>
+        <v>44</v>
       </c>
     </row>
     <row r="20" spans="1:39" x14ac:dyDescent="0.3">
@@ -4421,7 +4484,7 @@
         <v>39</v>
       </c>
       <c r="B20" t="s">
-        <v>283</v>
+        <v>274</v>
       </c>
       <c r="C20" t="s">
         <v>41</v>
@@ -4436,22 +4499,22 @@
         <v>44</v>
       </c>
       <c r="G20" t="s">
-        <v>284</v>
+        <v>69</v>
       </c>
       <c r="H20" t="s">
-        <v>285</v>
+        <v>275</v>
       </c>
       <c r="I20" t="s">
-        <v>203</v>
+        <v>47</v>
       </c>
       <c r="J20" t="s">
-        <v>286</v>
+        <v>276</v>
       </c>
       <c r="K20" t="s">
-        <v>287</v>
+        <v>277</v>
       </c>
       <c r="L20" t="s">
-        <v>288</v>
+        <v>278</v>
       </c>
       <c r="M20" t="s">
         <v>51</v>
@@ -4460,52 +4523,52 @@
         <v>52</v>
       </c>
       <c r="O20" t="s">
-        <v>289</v>
+        <v>53</v>
       </c>
       <c r="P20" t="s">
-        <v>44</v>
+        <v>279</v>
       </c>
       <c r="Q20" t="s">
-        <v>290</v>
+        <v>279</v>
       </c>
       <c r="R20" t="s">
-        <v>291</v>
+        <v>280</v>
       </c>
       <c r="S20" t="s">
-        <v>244</v>
+        <v>264</v>
       </c>
       <c r="T20" t="s">
-        <v>277</v>
+        <v>281</v>
       </c>
       <c r="U20" t="s">
-        <v>278</v>
+        <v>282</v>
       </c>
       <c r="V20" t="s">
         <v>57</v>
       </c>
       <c r="W20" t="s">
-        <v>279</v>
+        <v>283</v>
       </c>
       <c r="X20" t="s">
-        <v>292</v>
+        <v>268</v>
       </c>
       <c r="Y20" t="s">
-        <v>60</v>
+        <v>284</v>
       </c>
       <c r="Z20" t="s">
-        <v>42</v>
+        <v>285</v>
       </c>
       <c r="AA20" t="s">
-        <v>42</v>
+        <v>189</v>
       </c>
       <c r="AB20" t="s">
-        <v>279</v>
+        <v>286</v>
       </c>
       <c r="AC20" t="s">
-        <v>279</v>
+        <v>286</v>
       </c>
       <c r="AD20" t="s">
-        <v>293</v>
+        <v>287</v>
       </c>
       <c r="AE20" t="s">
         <v>63</v>
@@ -4514,22 +4577,22 @@
         <v>64</v>
       </c>
       <c r="AG20" t="s">
-        <v>294</v>
+        <v>288</v>
       </c>
       <c r="AH20" t="s">
-        <v>126</v>
+        <v>66</v>
       </c>
       <c r="AI20" t="s">
-        <v>127</v>
+        <v>67</v>
       </c>
       <c r="AJ20" t="s">
         <v>44</v>
       </c>
       <c r="AK20" t="s">
-        <v>252</v>
+        <v>272</v>
       </c>
       <c r="AL20" t="s">
-        <v>253</v>
+        <v>273</v>
       </c>
       <c r="AM20" t="s">
         <v>44</v>
@@ -4540,7 +4603,7 @@
         <v>39</v>
       </c>
       <c r="B21" t="s">
-        <v>295</v>
+        <v>289</v>
       </c>
       <c r="C21" t="s">
         <v>41</v>
@@ -4549,28 +4612,28 @@
         <v>42</v>
       </c>
       <c r="E21" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="F21" t="s">
         <v>44</v>
       </c>
       <c r="G21" t="s">
-        <v>44</v>
+        <v>290</v>
       </c>
       <c r="H21" t="s">
-        <v>296</v>
+        <v>291</v>
       </c>
       <c r="I21" t="s">
-        <v>203</v>
+        <v>224</v>
       </c>
       <c r="J21" t="s">
-        <v>297</v>
+        <v>292</v>
       </c>
       <c r="K21" t="s">
-        <v>298</v>
+        <v>293</v>
       </c>
       <c r="L21" t="s">
-        <v>299</v>
+        <v>294</v>
       </c>
       <c r="M21" t="s">
         <v>51</v>
@@ -4579,76 +4642,76 @@
         <v>52</v>
       </c>
       <c r="O21" t="s">
-        <v>300</v>
+        <v>295</v>
       </c>
       <c r="P21" t="s">
-        <v>301</v>
+        <v>44</v>
       </c>
       <c r="Q21" t="s">
-        <v>302</v>
+        <v>296</v>
       </c>
       <c r="R21" t="s">
-        <v>303</v>
+        <v>297</v>
       </c>
       <c r="S21" t="s">
-        <v>244</v>
+        <v>264</v>
       </c>
       <c r="T21" t="s">
-        <v>277</v>
+        <v>298</v>
       </c>
       <c r="U21" t="s">
-        <v>278</v>
+        <v>299</v>
       </c>
       <c r="V21" t="s">
         <v>57</v>
       </c>
       <c r="W21" t="s">
-        <v>279</v>
+        <v>300</v>
       </c>
       <c r="X21" t="s">
+        <v>301</v>
+      </c>
+      <c r="Y21" t="s">
+        <v>60</v>
+      </c>
+      <c r="Z21" t="s">
         <v>42</v>
       </c>
-      <c r="Y21" t="s">
+      <c r="AA21" t="s">
         <v>42</v>
       </c>
-      <c r="Z21" t="s">
-        <v>304</v>
-      </c>
-      <c r="AA21" t="s">
-        <v>305</v>
-      </c>
       <c r="AB21" t="s">
-        <v>306</v>
+        <v>300</v>
       </c>
       <c r="AC21" t="s">
-        <v>306</v>
+        <v>300</v>
       </c>
       <c r="AD21" t="s">
-        <v>306</v>
+        <v>302</v>
       </c>
       <c r="AE21" t="s">
         <v>63</v>
       </c>
       <c r="AF21" t="s">
-        <v>307</v>
+        <v>64</v>
       </c>
       <c r="AG21" t="s">
-        <v>306</v>
+        <v>303</v>
       </c>
       <c r="AH21" t="s">
-        <v>173</v>
+        <v>137</v>
       </c>
       <c r="AI21" t="s">
-        <v>308</v>
+        <v>138</v>
       </c>
       <c r="AJ21" t="s">
         <v>44</v>
       </c>
       <c r="AK21" t="s">
-        <v>252</v>
+        <v>272</v>
       </c>
       <c r="AL21" t="s">
-        <v>253</v>
+        <v>273</v>
       </c>
       <c r="AM21" t="s">
         <v>44</v>
@@ -4659,7 +4722,7 @@
         <v>39</v>
       </c>
       <c r="B22" t="s">
-        <v>309</v>
+        <v>304</v>
       </c>
       <c r="C22" t="s">
         <v>41</v>
@@ -4668,106 +4731,106 @@
         <v>42</v>
       </c>
       <c r="E22" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="F22" t="s">
         <v>44</v>
       </c>
       <c r="G22" t="s">
-        <v>69</v>
+        <v>44</v>
       </c>
       <c r="H22" t="s">
-        <v>107</v>
+        <v>305</v>
       </c>
       <c r="I22" t="s">
-        <v>130</v>
+        <v>224</v>
       </c>
       <c r="J22" t="s">
-        <v>310</v>
+        <v>306</v>
       </c>
       <c r="K22" t="s">
-        <v>311</v>
+        <v>307</v>
       </c>
       <c r="L22" t="s">
-        <v>312</v>
+        <v>308</v>
       </c>
       <c r="M22" t="s">
         <v>51</v>
       </c>
       <c r="N22" t="s">
-        <v>184</v>
+        <v>52</v>
       </c>
       <c r="O22" t="s">
-        <v>185</v>
+        <v>309</v>
       </c>
       <c r="P22" t="s">
-        <v>313</v>
+        <v>310</v>
       </c>
       <c r="Q22" t="s">
-        <v>313</v>
+        <v>311</v>
       </c>
       <c r="R22" t="s">
-        <v>314</v>
+        <v>312</v>
       </c>
       <c r="S22" t="s">
-        <v>244</v>
+        <v>264</v>
       </c>
       <c r="T22" t="s">
-        <v>261</v>
+        <v>298</v>
       </c>
       <c r="U22" t="s">
-        <v>262</v>
+        <v>299</v>
       </c>
       <c r="V22" t="s">
         <v>57</v>
       </c>
       <c r="W22" t="s">
-        <v>263</v>
+        <v>300</v>
       </c>
       <c r="X22" t="s">
-        <v>248</v>
+        <v>42</v>
       </c>
       <c r="Y22" t="s">
-        <v>264</v>
+        <v>42</v>
       </c>
       <c r="Z22" t="s">
-        <v>265</v>
+        <v>313</v>
       </c>
       <c r="AA22" t="s">
-        <v>178</v>
+        <v>314</v>
       </c>
       <c r="AB22" t="s">
-        <v>266</v>
+        <v>315</v>
       </c>
       <c r="AC22" t="s">
-        <v>266</v>
+        <v>315</v>
       </c>
       <c r="AD22" t="s">
-        <v>267</v>
+        <v>315</v>
       </c>
       <c r="AE22" t="s">
         <v>63</v>
       </c>
       <c r="AF22" t="s">
-        <v>102</v>
+        <v>316</v>
       </c>
       <c r="AG22" t="s">
         <v>315</v>
       </c>
       <c r="AH22" t="s">
-        <v>89</v>
+        <v>184</v>
       </c>
       <c r="AI22" t="s">
-        <v>136</v>
+        <v>317</v>
       </c>
       <c r="AJ22" t="s">
         <v>44</v>
       </c>
       <c r="AK22" t="s">
-        <v>252</v>
+        <v>272</v>
       </c>
       <c r="AL22" t="s">
-        <v>253</v>
+        <v>273</v>
       </c>
       <c r="AM22" t="s">
         <v>44</v>
@@ -4778,7 +4841,7 @@
         <v>39</v>
       </c>
       <c r="B23" t="s">
-        <v>316</v>
+        <v>318</v>
       </c>
       <c r="C23" t="s">
         <v>41</v>
@@ -4787,106 +4850,106 @@
         <v>42</v>
       </c>
       <c r="E23" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="F23" t="s">
         <v>44</v>
       </c>
       <c r="G23" t="s">
-        <v>44</v>
+        <v>69</v>
       </c>
       <c r="H23" t="s">
-        <v>296</v>
+        <v>107</v>
       </c>
       <c r="I23" t="s">
-        <v>203</v>
+        <v>141</v>
       </c>
       <c r="J23" t="s">
-        <v>317</v>
+        <v>319</v>
       </c>
       <c r="K23" t="s">
-        <v>318</v>
+        <v>320</v>
       </c>
       <c r="L23" t="s">
-        <v>319</v>
+        <v>321</v>
       </c>
       <c r="M23" t="s">
         <v>51</v>
       </c>
       <c r="N23" t="s">
-        <v>52</v>
+        <v>195</v>
       </c>
       <c r="O23" t="s">
-        <v>320</v>
+        <v>196</v>
       </c>
       <c r="P23" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="Q23" t="s">
-        <v>321</v>
+        <v>322</v>
       </c>
       <c r="R23" t="s">
-        <v>322</v>
+        <v>323</v>
       </c>
       <c r="S23" t="s">
-        <v>244</v>
+        <v>264</v>
       </c>
       <c r="T23" t="s">
-        <v>261</v>
+        <v>281</v>
       </c>
       <c r="U23" t="s">
-        <v>262</v>
+        <v>282</v>
       </c>
       <c r="V23" t="s">
         <v>57</v>
       </c>
       <c r="W23" t="s">
-        <v>263</v>
+        <v>283</v>
       </c>
       <c r="X23" t="s">
-        <v>42</v>
+        <v>268</v>
       </c>
       <c r="Y23" t="s">
-        <v>42</v>
+        <v>284</v>
       </c>
       <c r="Z23" t="s">
-        <v>323</v>
+        <v>285</v>
       </c>
       <c r="AA23" t="s">
-        <v>324</v>
+        <v>189</v>
       </c>
       <c r="AB23" t="s">
-        <v>325</v>
+        <v>286</v>
       </c>
       <c r="AC23" t="s">
-        <v>325</v>
+        <v>286</v>
       </c>
       <c r="AD23" t="s">
-        <v>325</v>
+        <v>287</v>
       </c>
       <c r="AE23" t="s">
         <v>63</v>
       </c>
       <c r="AF23" t="s">
-        <v>307</v>
+        <v>102</v>
       </c>
       <c r="AG23" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="AH23" t="s">
-        <v>173</v>
+        <v>89</v>
       </c>
       <c r="AI23" t="s">
-        <v>308</v>
+        <v>147</v>
       </c>
       <c r="AJ23" t="s">
-        <v>326</v>
+        <v>44</v>
       </c>
       <c r="AK23" t="s">
-        <v>327</v>
+        <v>272</v>
       </c>
       <c r="AL23" t="s">
-        <v>328</v>
+        <v>273</v>
       </c>
       <c r="AM23" t="s">
         <v>44</v>
@@ -4897,7 +4960,7 @@
         <v>39</v>
       </c>
       <c r="B24" t="s">
-        <v>329</v>
+        <v>325</v>
       </c>
       <c r="C24" t="s">
         <v>41</v>
@@ -4906,28 +4969,28 @@
         <v>42</v>
       </c>
       <c r="E24" t="s">
-        <v>330</v>
+        <v>44</v>
       </c>
       <c r="F24" t="s">
-        <v>330</v>
+        <v>44</v>
       </c>
       <c r="G24" t="s">
-        <v>331</v>
+        <v>44</v>
       </c>
       <c r="H24" t="s">
-        <v>332</v>
+        <v>305</v>
       </c>
       <c r="I24" t="s">
-        <v>333</v>
+        <v>224</v>
       </c>
       <c r="J24" t="s">
-        <v>334</v>
+        <v>326</v>
       </c>
       <c r="K24" t="s">
-        <v>335</v>
+        <v>327</v>
       </c>
       <c r="L24" t="s">
-        <v>336</v>
+        <v>328</v>
       </c>
       <c r="M24" t="s">
         <v>51</v>
@@ -4936,76 +4999,76 @@
         <v>52</v>
       </c>
       <c r="O24" t="s">
-        <v>53</v>
+        <v>123</v>
       </c>
       <c r="P24" t="s">
-        <v>44</v>
+        <v>329</v>
       </c>
       <c r="Q24" t="s">
-        <v>337</v>
+        <v>329</v>
       </c>
       <c r="R24" t="s">
-        <v>338</v>
+        <v>330</v>
       </c>
       <c r="S24" t="s">
-        <v>244</v>
+        <v>264</v>
       </c>
       <c r="T24" t="s">
-        <v>261</v>
+        <v>281</v>
       </c>
       <c r="U24" t="s">
-        <v>262</v>
+        <v>282</v>
       </c>
       <c r="V24" t="s">
         <v>57</v>
       </c>
       <c r="W24" t="s">
-        <v>263</v>
+        <v>283</v>
       </c>
       <c r="X24" t="s">
-        <v>339</v>
+        <v>42</v>
       </c>
       <c r="Y24" t="s">
-        <v>340</v>
+        <v>42</v>
       </c>
       <c r="Z24" t="s">
-        <v>341</v>
+        <v>331</v>
       </c>
       <c r="AA24" t="s">
-        <v>173</v>
+        <v>332</v>
       </c>
       <c r="AB24" t="s">
-        <v>342</v>
+        <v>333</v>
       </c>
       <c r="AC24" t="s">
-        <v>342</v>
+        <v>333</v>
       </c>
       <c r="AD24" t="s">
-        <v>343</v>
+        <v>333</v>
       </c>
       <c r="AE24" t="s">
         <v>63</v>
       </c>
       <c r="AF24" t="s">
-        <v>188</v>
+        <v>316</v>
       </c>
       <c r="AG24" t="s">
-        <v>344</v>
+        <v>333</v>
       </c>
       <c r="AH24" t="s">
-        <v>89</v>
+        <v>184</v>
       </c>
       <c r="AI24" t="s">
-        <v>136</v>
+        <v>317</v>
       </c>
       <c r="AJ24" t="s">
-        <v>326</v>
+        <v>334</v>
       </c>
       <c r="AK24" t="s">
-        <v>345</v>
+        <v>335</v>
       </c>
       <c r="AL24" t="s">
-        <v>346</v>
+        <v>336</v>
       </c>
       <c r="AM24" t="s">
         <v>44</v>
@@ -5016,7 +5079,7 @@
         <v>39</v>
       </c>
       <c r="B25" t="s">
-        <v>347</v>
+        <v>337</v>
       </c>
       <c r="C25" t="s">
         <v>41</v>
@@ -5025,106 +5088,106 @@
         <v>42</v>
       </c>
       <c r="E25" t="s">
-        <v>43</v>
+        <v>338</v>
       </c>
       <c r="F25" t="s">
-        <v>44</v>
+        <v>338</v>
       </c>
       <c r="G25" t="s">
-        <v>69</v>
+        <v>339</v>
       </c>
       <c r="H25" t="s">
-        <v>348</v>
+        <v>340</v>
       </c>
       <c r="I25" t="s">
-        <v>130</v>
+        <v>341</v>
       </c>
       <c r="J25" t="s">
-        <v>349</v>
+        <v>342</v>
       </c>
       <c r="K25" t="s">
-        <v>350</v>
+        <v>343</v>
       </c>
       <c r="L25" t="s">
-        <v>351</v>
+        <v>344</v>
       </c>
       <c r="M25" t="s">
         <v>51</v>
       </c>
       <c r="N25" t="s">
-        <v>184</v>
+        <v>52</v>
       </c>
       <c r="O25" t="s">
-        <v>185</v>
+        <v>53</v>
       </c>
       <c r="P25" t="s">
-        <v>352</v>
+        <v>44</v>
       </c>
       <c r="Q25" t="s">
-        <v>352</v>
+        <v>345</v>
       </c>
       <c r="R25" t="s">
-        <v>353</v>
+        <v>346</v>
       </c>
       <c r="S25" t="s">
-        <v>244</v>
+        <v>264</v>
       </c>
       <c r="T25" t="s">
-        <v>245</v>
+        <v>281</v>
       </c>
       <c r="U25" t="s">
-        <v>246</v>
+        <v>282</v>
       </c>
       <c r="V25" t="s">
         <v>57</v>
       </c>
       <c r="W25" t="s">
-        <v>247</v>
+        <v>283</v>
       </c>
       <c r="X25" t="s">
-        <v>354</v>
+        <v>347</v>
       </c>
       <c r="Y25" t="s">
-        <v>87</v>
+        <v>348</v>
       </c>
       <c r="Z25" t="s">
-        <v>355</v>
+        <v>349</v>
       </c>
       <c r="AA25" t="s">
-        <v>173</v>
+        <v>184</v>
       </c>
       <c r="AB25" t="s">
-        <v>356</v>
+        <v>350</v>
       </c>
       <c r="AC25" t="s">
-        <v>356</v>
+        <v>350</v>
       </c>
       <c r="AD25" t="s">
-        <v>357</v>
+        <v>351</v>
       </c>
       <c r="AE25" t="s">
         <v>63</v>
       </c>
       <c r="AF25" t="s">
-        <v>102</v>
+        <v>199</v>
       </c>
       <c r="AG25" t="s">
-        <v>358</v>
+        <v>352</v>
       </c>
       <c r="AH25" t="s">
-        <v>359</v>
+        <v>89</v>
       </c>
       <c r="AI25" t="s">
-        <v>360</v>
+        <v>147</v>
       </c>
       <c r="AJ25" t="s">
-        <v>326</v>
+        <v>334</v>
       </c>
       <c r="AK25" t="s">
-        <v>361</v>
+        <v>353</v>
       </c>
       <c r="AL25" t="s">
-        <v>362</v>
+        <v>354</v>
       </c>
       <c r="AM25" t="s">
         <v>44</v>
@@ -5135,7 +5198,7 @@
         <v>39</v>
       </c>
       <c r="B26" t="s">
-        <v>363</v>
+        <v>355</v>
       </c>
       <c r="C26" t="s">
         <v>41</v>
@@ -5144,106 +5207,106 @@
         <v>42</v>
       </c>
       <c r="E26" t="s">
-        <v>364</v>
+        <v>43</v>
       </c>
       <c r="F26" t="s">
         <v>44</v>
       </c>
       <c r="G26" t="s">
-        <v>365</v>
+        <v>69</v>
       </c>
       <c r="H26" t="s">
-        <v>366</v>
+        <v>356</v>
       </c>
       <c r="I26" t="s">
-        <v>130</v>
+        <v>141</v>
       </c>
       <c r="J26" t="s">
-        <v>367</v>
+        <v>357</v>
       </c>
       <c r="K26" t="s">
-        <v>368</v>
+        <v>358</v>
       </c>
       <c r="L26" t="s">
-        <v>369</v>
+        <v>359</v>
       </c>
       <c r="M26" t="s">
         <v>51</v>
       </c>
       <c r="N26" t="s">
-        <v>52</v>
+        <v>195</v>
       </c>
       <c r="O26" t="s">
-        <v>370</v>
+        <v>196</v>
       </c>
       <c r="P26" t="s">
-        <v>44</v>
+        <v>360</v>
       </c>
       <c r="Q26" t="s">
-        <v>371</v>
+        <v>360</v>
       </c>
       <c r="R26" t="s">
-        <v>372</v>
+        <v>361</v>
       </c>
       <c r="S26" t="s">
-        <v>244</v>
+        <v>264</v>
       </c>
       <c r="T26" t="s">
-        <v>245</v>
+        <v>265</v>
       </c>
       <c r="U26" t="s">
-        <v>246</v>
+        <v>266</v>
       </c>
       <c r="V26" t="s">
         <v>57</v>
       </c>
       <c r="W26" t="s">
-        <v>247</v>
+        <v>267</v>
       </c>
       <c r="X26" t="s">
-        <v>59</v>
+        <v>362</v>
       </c>
       <c r="Y26" t="s">
         <v>87</v>
       </c>
       <c r="Z26" t="s">
-        <v>373</v>
+        <v>363</v>
       </c>
       <c r="AA26" t="s">
-        <v>374</v>
+        <v>184</v>
       </c>
       <c r="AB26" t="s">
-        <v>375</v>
+        <v>364</v>
       </c>
       <c r="AC26" t="s">
-        <v>375</v>
+        <v>364</v>
       </c>
       <c r="AD26" t="s">
-        <v>376</v>
+        <v>365</v>
       </c>
       <c r="AE26" t="s">
         <v>63</v>
       </c>
       <c r="AF26" t="s">
-        <v>377</v>
+        <v>102</v>
       </c>
       <c r="AG26" t="s">
-        <v>378</v>
+        <v>366</v>
       </c>
       <c r="AH26" t="s">
-        <v>173</v>
+        <v>367</v>
       </c>
       <c r="AI26" t="s">
-        <v>308</v>
+        <v>368</v>
       </c>
       <c r="AJ26" t="s">
-        <v>326</v>
+        <v>334</v>
       </c>
       <c r="AK26" t="s">
-        <v>379</v>
+        <v>369</v>
       </c>
       <c r="AL26" t="s">
-        <v>362</v>
+        <v>370</v>
       </c>
       <c r="AM26" t="s">
         <v>44</v>
@@ -5254,7 +5317,7 @@
         <v>39</v>
       </c>
       <c r="B27" t="s">
-        <v>380</v>
+        <v>371</v>
       </c>
       <c r="C27" t="s">
         <v>41</v>
@@ -5263,28 +5326,28 @@
         <v>42</v>
       </c>
       <c r="E27" t="s">
-        <v>43</v>
+        <v>372</v>
       </c>
       <c r="F27" t="s">
         <v>44</v>
       </c>
       <c r="G27" t="s">
-        <v>284</v>
+        <v>373</v>
       </c>
       <c r="H27" t="s">
-        <v>285</v>
+        <v>374</v>
       </c>
       <c r="I27" t="s">
-        <v>165</v>
+        <v>141</v>
       </c>
       <c r="J27" t="s">
-        <v>381</v>
+        <v>375</v>
       </c>
       <c r="K27" t="s">
-        <v>382</v>
+        <v>376</v>
       </c>
       <c r="L27" t="s">
-        <v>383</v>
+        <v>377</v>
       </c>
       <c r="M27" t="s">
         <v>51</v>
@@ -5293,76 +5356,76 @@
         <v>52</v>
       </c>
       <c r="O27" t="s">
-        <v>53</v>
+        <v>378</v>
       </c>
       <c r="P27" t="s">
         <v>44</v>
       </c>
       <c r="Q27" t="s">
-        <v>384</v>
+        <v>379</v>
       </c>
       <c r="R27" t="s">
-        <v>385</v>
+        <v>380</v>
       </c>
       <c r="S27" t="s">
-        <v>244</v>
+        <v>264</v>
       </c>
       <c r="T27" t="s">
-        <v>277</v>
+        <v>265</v>
       </c>
       <c r="U27" t="s">
-        <v>278</v>
+        <v>266</v>
       </c>
       <c r="V27" t="s">
         <v>57</v>
       </c>
       <c r="W27" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="X27" t="s">
-        <v>341</v>
+        <v>59</v>
       </c>
       <c r="Y27" t="s">
-        <v>60</v>
+        <v>87</v>
       </c>
       <c r="Z27" t="s">
-        <v>341</v>
+        <v>381</v>
       </c>
       <c r="AA27" t="s">
-        <v>173</v>
+        <v>382</v>
       </c>
       <c r="AB27" t="s">
-        <v>342</v>
+        <v>383</v>
       </c>
       <c r="AC27" t="s">
-        <v>342</v>
+        <v>383</v>
       </c>
       <c r="AD27" t="s">
-        <v>266</v>
+        <v>384</v>
       </c>
       <c r="AE27" t="s">
         <v>63</v>
       </c>
       <c r="AF27" t="s">
-        <v>102</v>
+        <v>385</v>
       </c>
       <c r="AG27" t="s">
         <v>386</v>
       </c>
       <c r="AH27" t="s">
+        <v>184</v>
+      </c>
+      <c r="AI27" t="s">
+        <v>317</v>
+      </c>
+      <c r="AJ27" t="s">
+        <v>334</v>
+      </c>
+      <c r="AK27" t="s">
         <v>387</v>
       </c>
-      <c r="AI27" t="s">
-        <v>388</v>
-      </c>
-      <c r="AJ27" t="s">
-        <v>326</v>
-      </c>
-      <c r="AK27" t="s">
-        <v>389</v>
-      </c>
       <c r="AL27" t="s">
-        <v>390</v>
+        <v>370</v>
       </c>
       <c r="AM27" t="s">
         <v>44</v>
@@ -5373,7 +5436,7 @@
         <v>39</v>
       </c>
       <c r="B28" t="s">
-        <v>391</v>
+        <v>388</v>
       </c>
       <c r="C28" t="s">
         <v>41</v>
@@ -5382,28 +5445,28 @@
         <v>42</v>
       </c>
       <c r="E28" t="s">
-        <v>330</v>
+        <v>43</v>
       </c>
       <c r="F28" t="s">
-        <v>330</v>
+        <v>44</v>
       </c>
       <c r="G28" t="s">
-        <v>331</v>
+        <v>45</v>
       </c>
       <c r="H28" t="s">
-        <v>332</v>
+        <v>46</v>
       </c>
       <c r="I28" t="s">
-        <v>165</v>
+        <v>119</v>
       </c>
       <c r="J28" t="s">
-        <v>392</v>
+        <v>389</v>
       </c>
       <c r="K28" t="s">
-        <v>393</v>
+        <v>390</v>
       </c>
       <c r="L28" t="s">
-        <v>394</v>
+        <v>391</v>
       </c>
       <c r="M28" t="s">
         <v>51</v>
@@ -5412,37 +5475,37 @@
         <v>52</v>
       </c>
       <c r="O28" t="s">
-        <v>53</v>
+        <v>392</v>
       </c>
       <c r="P28" t="s">
         <v>44</v>
       </c>
       <c r="Q28" t="s">
-        <v>395</v>
+        <v>393</v>
       </c>
       <c r="R28" t="s">
-        <v>396</v>
+        <v>394</v>
       </c>
       <c r="S28" t="s">
-        <v>244</v>
+        <v>264</v>
       </c>
       <c r="T28" t="s">
-        <v>277</v>
+        <v>298</v>
       </c>
       <c r="U28" t="s">
-        <v>278</v>
+        <v>299</v>
       </c>
       <c r="V28" t="s">
         <v>57</v>
       </c>
       <c r="W28" t="s">
-        <v>263</v>
+        <v>300</v>
       </c>
       <c r="X28" t="s">
-        <v>397</v>
+        <v>395</v>
       </c>
       <c r="Y28" t="s">
-        <v>398</v>
+        <v>60</v>
       </c>
       <c r="Z28" t="s">
         <v>42</v>
@@ -5451,37 +5514,37 @@
         <v>42</v>
       </c>
       <c r="AB28" t="s">
-        <v>263</v>
+        <v>300</v>
       </c>
       <c r="AC28" t="s">
-        <v>263</v>
+        <v>300</v>
       </c>
       <c r="AD28" t="s">
-        <v>399</v>
+        <v>396</v>
       </c>
       <c r="AE28" t="s">
         <v>63</v>
       </c>
       <c r="AF28" t="s">
-        <v>377</v>
+        <v>64</v>
       </c>
       <c r="AG28" t="s">
+        <v>397</v>
+      </c>
+      <c r="AH28" t="s">
+        <v>398</v>
+      </c>
+      <c r="AI28" t="s">
+        <v>399</v>
+      </c>
+      <c r="AJ28" t="s">
+        <v>334</v>
+      </c>
+      <c r="AK28" t="s">
         <v>400</v>
       </c>
-      <c r="AH28" t="s">
-        <v>307</v>
-      </c>
-      <c r="AI28" t="s">
+      <c r="AL28" t="s">
         <v>401</v>
-      </c>
-      <c r="AJ28" t="s">
-        <v>326</v>
-      </c>
-      <c r="AK28" t="s">
-        <v>402</v>
-      </c>
-      <c r="AL28" t="s">
-        <v>390</v>
       </c>
       <c r="AM28" t="s">
         <v>44</v>
@@ -5492,37 +5555,37 @@
         <v>39</v>
       </c>
       <c r="B29" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="C29" t="s">
         <v>41</v>
       </c>
       <c r="D29" t="s">
+        <v>42</v>
+      </c>
+      <c r="E29" t="s">
+        <v>43</v>
+      </c>
+      <c r="F29" t="s">
+        <v>44</v>
+      </c>
+      <c r="G29" t="s">
+        <v>290</v>
+      </c>
+      <c r="H29" t="s">
+        <v>291</v>
+      </c>
+      <c r="I29" t="s">
+        <v>176</v>
+      </c>
+      <c r="J29" t="s">
+        <v>403</v>
+      </c>
+      <c r="K29" t="s">
         <v>404</v>
       </c>
-      <c r="E29" t="s">
+      <c r="L29" t="s">
         <v>405</v>
-      </c>
-      <c r="F29" t="s">
-        <v>365</v>
-      </c>
-      <c r="G29" t="s">
-        <v>406</v>
-      </c>
-      <c r="H29" t="s">
-        <v>406</v>
-      </c>
-      <c r="I29" t="s">
-        <v>44</v>
-      </c>
-      <c r="J29" t="s">
-        <v>407</v>
-      </c>
-      <c r="K29" t="s">
-        <v>408</v>
-      </c>
-      <c r="L29" t="s">
-        <v>409</v>
       </c>
       <c r="M29" t="s">
         <v>51</v>
@@ -5531,79 +5594,317 @@
         <v>52</v>
       </c>
       <c r="O29" t="s">
-        <v>410</v>
+        <v>53</v>
       </c>
       <c r="P29" t="s">
         <v>44</v>
       </c>
       <c r="Q29" t="s">
-        <v>411</v>
+        <v>406</v>
       </c>
       <c r="R29" t="s">
-        <v>412</v>
+        <v>407</v>
       </c>
       <c r="S29" t="s">
-        <v>413</v>
+        <v>264</v>
       </c>
       <c r="T29" t="s">
-        <v>414</v>
+        <v>298</v>
       </c>
       <c r="U29" t="s">
-        <v>415</v>
+        <v>299</v>
       </c>
       <c r="V29" t="s">
         <v>57</v>
       </c>
       <c r="W29" t="s">
-        <v>416</v>
+        <v>283</v>
       </c>
       <c r="X29" t="s">
-        <v>404</v>
+        <v>349</v>
       </c>
       <c r="Y29" t="s">
         <v>60</v>
       </c>
       <c r="Z29" t="s">
+        <v>349</v>
+      </c>
+      <c r="AA29" t="s">
+        <v>184</v>
+      </c>
+      <c r="AB29" t="s">
+        <v>350</v>
+      </c>
+      <c r="AC29" t="s">
+        <v>350</v>
+      </c>
+      <c r="AD29" t="s">
+        <v>286</v>
+      </c>
+      <c r="AE29" t="s">
+        <v>63</v>
+      </c>
+      <c r="AF29" t="s">
+        <v>102</v>
+      </c>
+      <c r="AG29" t="s">
+        <v>408</v>
+      </c>
+      <c r="AH29" t="s">
+        <v>398</v>
+      </c>
+      <c r="AI29" t="s">
+        <v>409</v>
+      </c>
+      <c r="AJ29" t="s">
+        <v>334</v>
+      </c>
+      <c r="AK29" t="s">
+        <v>410</v>
+      </c>
+      <c r="AL29" t="s">
+        <v>411</v>
+      </c>
+      <c r="AM29" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="30" spans="1:39" x14ac:dyDescent="0.3">
+      <c r="A30" t="s">
+        <v>39</v>
+      </c>
+      <c r="B30" t="s">
+        <v>412</v>
+      </c>
+      <c r="C30" t="s">
+        <v>41</v>
+      </c>
+      <c r="D30" t="s">
+        <v>42</v>
+      </c>
+      <c r="E30" t="s">
+        <v>338</v>
+      </c>
+      <c r="F30" t="s">
+        <v>338</v>
+      </c>
+      <c r="G30" t="s">
+        <v>339</v>
+      </c>
+      <c r="H30" t="s">
+        <v>340</v>
+      </c>
+      <c r="I30" t="s">
+        <v>176</v>
+      </c>
+      <c r="J30" t="s">
+        <v>413</v>
+      </c>
+      <c r="K30" t="s">
+        <v>414</v>
+      </c>
+      <c r="L30" t="s">
+        <v>415</v>
+      </c>
+      <c r="M30" t="s">
+        <v>51</v>
+      </c>
+      <c r="N30" t="s">
+        <v>52</v>
+      </c>
+      <c r="O30" t="s">
+        <v>53</v>
+      </c>
+      <c r="P30" t="s">
+        <v>44</v>
+      </c>
+      <c r="Q30" t="s">
+        <v>416</v>
+      </c>
+      <c r="R30" t="s">
         <v>417</v>
       </c>
-      <c r="AA29" t="s">
-        <v>210</v>
-      </c>
-      <c r="AB29" t="s">
+      <c r="S30" t="s">
+        <v>264</v>
+      </c>
+      <c r="T30" t="s">
+        <v>298</v>
+      </c>
+      <c r="U30" t="s">
+        <v>299</v>
+      </c>
+      <c r="V30" t="s">
+        <v>57</v>
+      </c>
+      <c r="W30" t="s">
+        <v>283</v>
+      </c>
+      <c r="X30" t="s">
         <v>418</v>
       </c>
-      <c r="AC29" t="s">
-        <v>418</v>
-      </c>
-      <c r="AD29" t="s">
+      <c r="Y30" t="s">
         <v>419</v>
       </c>
-      <c r="AE29" t="s">
-        <v>44</v>
-      </c>
-      <c r="AF29" t="s">
+      <c r="Z30" t="s">
+        <v>42</v>
+      </c>
+      <c r="AA30" t="s">
+        <v>42</v>
+      </c>
+      <c r="AB30" t="s">
+        <v>283</v>
+      </c>
+      <c r="AC30" t="s">
+        <v>283</v>
+      </c>
+      <c r="AD30" t="s">
+        <v>420</v>
+      </c>
+      <c r="AE30" t="s">
+        <v>63</v>
+      </c>
+      <c r="AF30" t="s">
+        <v>385</v>
+      </c>
+      <c r="AG30" t="s">
+        <v>421</v>
+      </c>
+      <c r="AH30" t="s">
+        <v>316</v>
+      </c>
+      <c r="AI30" t="s">
+        <v>422</v>
+      </c>
+      <c r="AJ30" t="s">
+        <v>334</v>
+      </c>
+      <c r="AK30" t="s">
+        <v>423</v>
+      </c>
+      <c r="AL30" t="s">
+        <v>411</v>
+      </c>
+      <c r="AM30" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="31" spans="1:39" x14ac:dyDescent="0.3">
+      <c r="A31" t="s">
+        <v>39</v>
+      </c>
+      <c r="B31" t="s">
+        <v>424</v>
+      </c>
+      <c r="C31" t="s">
+        <v>41</v>
+      </c>
+      <c r="D31" t="s">
+        <v>425</v>
+      </c>
+      <c r="E31" t="s">
+        <v>426</v>
+      </c>
+      <c r="F31" t="s">
+        <v>373</v>
+      </c>
+      <c r="G31" t="s">
+        <v>427</v>
+      </c>
+      <c r="H31" t="s">
+        <v>427</v>
+      </c>
+      <c r="I31" t="s">
+        <v>44</v>
+      </c>
+      <c r="J31" t="s">
+        <v>428</v>
+      </c>
+      <c r="K31" t="s">
+        <v>429</v>
+      </c>
+      <c r="L31" t="s">
+        <v>430</v>
+      </c>
+      <c r="M31" t="s">
+        <v>51</v>
+      </c>
+      <c r="N31" t="s">
+        <v>52</v>
+      </c>
+      <c r="O31" t="s">
+        <v>431</v>
+      </c>
+      <c r="P31" t="s">
+        <v>44</v>
+      </c>
+      <c r="Q31" t="s">
+        <v>432</v>
+      </c>
+      <c r="R31" t="s">
+        <v>433</v>
+      </c>
+      <c r="S31" t="s">
+        <v>434</v>
+      </c>
+      <c r="T31" t="s">
+        <v>435</v>
+      </c>
+      <c r="U31" t="s">
+        <v>436</v>
+      </c>
+      <c r="V31" t="s">
+        <v>57</v>
+      </c>
+      <c r="W31" t="s">
+        <v>437</v>
+      </c>
+      <c r="X31" t="s">
+        <v>425</v>
+      </c>
+      <c r="Y31" t="s">
+        <v>60</v>
+      </c>
+      <c r="Z31" t="s">
+        <v>438</v>
+      </c>
+      <c r="AA31" t="s">
+        <v>231</v>
+      </c>
+      <c r="AB31" t="s">
+        <v>439</v>
+      </c>
+      <c r="AC31" t="s">
+        <v>439</v>
+      </c>
+      <c r="AD31" t="s">
+        <v>440</v>
+      </c>
+      <c r="AE31" t="s">
+        <v>44</v>
+      </c>
+      <c r="AF31" t="s">
         <v>93</v>
       </c>
-      <c r="AG29" t="s">
-        <v>420</v>
-      </c>
-      <c r="AH29" t="s">
-        <v>178</v>
-      </c>
-      <c r="AI29" t="s">
-        <v>179</v>
-      </c>
-      <c r="AJ29" t="s">
-        <v>326</v>
-      </c>
-      <c r="AK29" t="s">
-        <v>421</v>
-      </c>
-      <c r="AL29" t="s">
-        <v>390</v>
-      </c>
-      <c r="AM29" t="s">
-        <v>422</v>
+      <c r="AG31" t="s">
+        <v>441</v>
+      </c>
+      <c r="AH31" t="s">
+        <v>189</v>
+      </c>
+      <c r="AI31" t="s">
+        <v>190</v>
+      </c>
+      <c r="AJ31" t="s">
+        <v>334</v>
+      </c>
+      <c r="AK31" t="s">
+        <v>442</v>
+      </c>
+      <c r="AL31" t="s">
+        <v>411</v>
+      </c>
+      <c r="AM31" t="s">
+        <v>443</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
📊 Actualizar Abono_VU.xlsx — 26-03-2026, 11:54:34 a. m.
</commit_message>
<xml_diff>
--- a/datos/Abono_VU.xlsx
+++ b/datos/Abono_VU.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://funerariaimchile-my.sharepoint.com/personal/anais_gonzalez_funerariaim_cl/Documents/Dashboard_Control Diario de Ventas/Archivos diarios/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A6BFC294-D65A-4329-A3C7-0A7FC2987227}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{E1A0A991-7464-4500-BBBD-980D2D4C4263}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1209" uniqueCount="444">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1404" uniqueCount="501">
   <si>
     <t>EMPRESA</t>
   </si>
@@ -625,6 +625,81 @@
     <t>225000</t>
   </si>
   <si>
+    <t>1015683</t>
+  </si>
+  <si>
+    <t>Nayaret Tatiana Puga Marchant</t>
+  </si>
+  <si>
+    <t>25/03/2026</t>
+  </si>
+  <si>
+    <t>HERMOSILLA NORAMBUENA GRACIELA DEL CARMEN</t>
+  </si>
+  <si>
+    <t>6839198-9</t>
+  </si>
+  <si>
+    <t>La exótica  11122, La Pintana, Santiago, Metropolitana  Casa:</t>
+  </si>
+  <si>
+    <t>La Pintana</t>
+  </si>
+  <si>
+    <t>987418795</t>
+  </si>
+  <si>
+    <t>mana2010@live.cl</t>
+  </si>
+  <si>
+    <t>1000000</t>
+  </si>
+  <si>
+    <t>2000000</t>
+  </si>
+  <si>
+    <t>33916</t>
+  </si>
+  <si>
+    <t>21</t>
+  </si>
+  <si>
+    <t>21/04/2026</t>
+  </si>
+  <si>
+    <t>1015668</t>
+  </si>
+  <si>
+    <t>ANDREA VALESKA SAFFA ROMERO</t>
+  </si>
+  <si>
+    <t>CARRASCO HERNANDEZ MARTA</t>
+  </si>
+  <si>
+    <t>8626435-8</t>
+  </si>
+  <si>
+    <t>Pasaje pullay, ALT 5838 - Renca -</t>
+  </si>
+  <si>
+    <t>Renca</t>
+  </si>
+  <si>
+    <t>954940199</t>
+  </si>
+  <si>
+    <t>936883029</t>
+  </si>
+  <si>
+    <t>jessica.carrasco46@gmail.com</t>
+  </si>
+  <si>
+    <t>2521008.403</t>
+  </si>
+  <si>
+    <t>2026-03-25T00:00:00</t>
+  </si>
+  <si>
     <t>1015622</t>
   </si>
   <si>
@@ -661,9 +736,6 @@
     <t>1015684</t>
   </si>
   <si>
-    <t>Nayaret Tatiana Puga Marchant</t>
-  </si>
-  <si>
     <t>GUERRA LEIVA ANA EDELMIRA</t>
   </si>
   <si>
@@ -997,6 +1069,51 @@
     <t>59847</t>
   </si>
   <si>
+    <t>1015685</t>
+  </si>
+  <si>
+    <t>130000</t>
+  </si>
+  <si>
+    <t>MILLAN LEVIO ELENA FRESIA</t>
+  </si>
+  <si>
+    <t>10483632-1</t>
+  </si>
+  <si>
+    <t>manuel busto 0451, ALT 451 - Quilicura -</t>
+  </si>
+  <si>
+    <t>937231044</t>
+  </si>
+  <si>
+    <t>elenamillanlevio64@gmail.com</t>
+  </si>
+  <si>
+    <t>72</t>
+  </si>
+  <si>
+    <t>49888.88</t>
+  </si>
+  <si>
+    <t>9</t>
+  </si>
+  <si>
+    <t>09/05/2026</t>
+  </si>
+  <si>
+    <t>3</t>
+  </si>
+  <si>
+    <t>3-AT-43</t>
+  </si>
+  <si>
+    <t>Valle de la Memoria</t>
+  </si>
+  <si>
+    <t>2025-10-31T00:00:00</t>
+  </si>
+  <si>
     <t>1015629</t>
   </si>
   <si>
@@ -1021,30 +1138,66 @@
     <t>79.96</t>
   </si>
   <si>
-    <t>1000000</t>
-  </si>
-  <si>
-    <t>3</t>
-  </si>
-  <si>
     <t>3-BA-43</t>
   </si>
   <si>
-    <t>Valle de la Memoria</t>
+    <t>1015692</t>
+  </si>
+  <si>
+    <t>340000</t>
+  </si>
+  <si>
+    <t>ERNESTO OLIVA</t>
+  </si>
+  <si>
+    <t>MIGUEL SANDOVAL</t>
+  </si>
+  <si>
+    <t>ANDREA CONCHA ADASME</t>
+  </si>
+  <si>
+    <t>ROSAS PALOMINOS MARISELA ELIZABETH</t>
+  </si>
+  <si>
+    <t>20.033.453-1</t>
+  </si>
+  <si>
+    <t>Estadio nacional , ALT 87 - Quilicura -</t>
+  </si>
+  <si>
+    <t>994955673</t>
+  </si>
+  <si>
+    <t>rosasmarisela382@gmail.com</t>
+  </si>
+  <si>
+    <t>500000</t>
+  </si>
+  <si>
+    <t>499000</t>
+  </si>
+  <si>
+    <t>4491000</t>
+  </si>
+  <si>
+    <t>3991000</t>
+  </si>
+  <si>
+    <t>66516.66</t>
+  </si>
+  <si>
+    <t>4</t>
+  </si>
+  <si>
+    <t>4-F-39</t>
+  </si>
+  <si>
+    <t>Valle de la Memoria 2</t>
   </si>
   <si>
     <t>1015647</t>
   </si>
   <si>
-    <t>ERNESTO OLIVA</t>
-  </si>
-  <si>
-    <t>MIGUEL SANDOVAL</t>
-  </si>
-  <si>
-    <t>ANDREA CONCHA ADASME</t>
-  </si>
-  <si>
     <t>17/03/2026</t>
   </si>
   <si>
@@ -1069,12 +1222,6 @@
     <t>0.26</t>
   </si>
   <si>
-    <t>499000</t>
-  </si>
-  <si>
-    <t>4491000</t>
-  </si>
-  <si>
     <t>3191000</t>
   </si>
   <si>
@@ -1084,9 +1231,6 @@
     <t>4-Z-42</t>
   </si>
   <si>
-    <t>Valle de la Memoria 2</t>
-  </si>
-  <si>
     <t>1015610</t>
   </si>
   <si>
@@ -1123,9 +1267,6 @@
     <t>46575</t>
   </si>
   <si>
-    <t>4</t>
-  </si>
-  <si>
     <t>04/04/2026</t>
   </si>
   <si>
@@ -1177,9 +1318,6 @@
     <t>2532000</t>
   </si>
   <si>
-    <t>72</t>
-  </si>
-  <si>
     <t>35143</t>
   </si>
   <si>
@@ -1198,9 +1336,6 @@
     <t>Antonio Maceo 3176, ALT 3176 - Renca -</t>
   </si>
   <si>
-    <t>Renca</t>
-  </si>
-  <si>
     <t>933158189</t>
   </si>
   <si>
@@ -1228,6 +1363,48 @@
     <t>Valles De las Rosas</t>
   </si>
   <si>
+    <t>1015686</t>
+  </si>
+  <si>
+    <t>449853.97</t>
+  </si>
+  <si>
+    <t>GALLARDO CONTRERAS SILVIA ISABEL</t>
+  </si>
+  <si>
+    <t>10740648-4</t>
+  </si>
+  <si>
+    <t>LOS ROBLES 485, ALT 485 - Quilicura -</t>
+  </si>
+  <si>
+    <t>964469773</t>
+  </si>
+  <si>
+    <t>975782194</t>
+  </si>
+  <si>
+    <t>sigallardo28@hotmail.com</t>
+  </si>
+  <si>
+    <t>0.34</t>
+  </si>
+  <si>
+    <t>3880000</t>
+  </si>
+  <si>
+    <t>107770</t>
+  </si>
+  <si>
+    <t>6</t>
+  </si>
+  <si>
+    <t>2-AA-4</t>
+  </si>
+  <si>
+    <t>Valles de Las Rosas 2</t>
+  </si>
+  <si>
     <t>1015620</t>
   </si>
   <si>
@@ -1255,9 +1432,6 @@
     <t>2-AH-15</t>
   </si>
   <si>
-    <t>Valles de Las Rosas 2</t>
-  </si>
-  <si>
     <t>1015605</t>
   </si>
   <si>
@@ -1295,9 +1469,6 @@
   </si>
   <si>
     <t>1015634</t>
-  </si>
-  <si>
-    <t>2000000</t>
   </si>
   <si>
     <t>GERENCIA DISTRITO 2</t>
@@ -2212,7 +2383,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AM31"/>
+  <dimension ref="A1:AM36"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="39" width="8" customWidth="1"/>
@@ -3791,16 +3962,16 @@
         <v>202</v>
       </c>
       <c r="I14" t="s">
-        <v>176</v>
+        <v>203</v>
       </c>
       <c r="J14" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="K14" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="L14" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="M14" t="s">
         <v>51</v>
@@ -3809,67 +3980,67 @@
         <v>52</v>
       </c>
       <c r="O14" t="s">
-        <v>53</v>
+        <v>207</v>
       </c>
       <c r="P14" t="s">
         <v>44</v>
       </c>
       <c r="Q14" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="R14" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="S14" t="s">
         <v>44</v>
       </c>
       <c r="T14" t="s">
-        <v>165</v>
+        <v>56</v>
       </c>
       <c r="U14" t="s">
-        <v>165</v>
+        <v>56</v>
       </c>
       <c r="V14" t="s">
         <v>57</v>
       </c>
       <c r="W14" t="s">
-        <v>166</v>
+        <v>58</v>
       </c>
       <c r="X14" t="s">
-        <v>183</v>
+        <v>210</v>
       </c>
       <c r="Y14" t="s">
-        <v>60</v>
+        <v>168</v>
       </c>
       <c r="Z14" t="s">
-        <v>183</v>
+        <v>42</v>
       </c>
       <c r="AA14" t="s">
-        <v>184</v>
+        <v>42</v>
       </c>
       <c r="AB14" t="s">
-        <v>185</v>
+        <v>58</v>
       </c>
       <c r="AC14" t="s">
-        <v>186</v>
+        <v>61</v>
       </c>
       <c r="AD14" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="AE14" t="s">
         <v>63</v>
       </c>
       <c r="AF14" t="s">
-        <v>93</v>
+        <v>126</v>
       </c>
       <c r="AG14" t="s">
-        <v>209</v>
+        <v>212</v>
       </c>
       <c r="AH14" t="s">
-        <v>210</v>
+        <v>213</v>
       </c>
       <c r="AI14" t="s">
-        <v>211</v>
+        <v>214</v>
       </c>
       <c r="AJ14" t="s">
         <v>44</v>
@@ -3889,13 +4060,13 @@
         <v>39</v>
       </c>
       <c r="B15" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="C15" t="s">
-        <v>41</v>
+        <v>130</v>
       </c>
       <c r="D15" t="s">
-        <v>42</v>
+        <v>59</v>
       </c>
       <c r="E15" t="s">
         <v>43</v>
@@ -3904,22 +4075,22 @@
         <v>44</v>
       </c>
       <c r="G15" t="s">
-        <v>77</v>
+        <v>69</v>
       </c>
       <c r="H15" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="I15" t="s">
-        <v>119</v>
+        <v>44</v>
       </c>
       <c r="J15" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
       <c r="K15" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="L15" t="s">
-        <v>216</v>
+        <v>219</v>
       </c>
       <c r="M15" t="s">
         <v>51</v>
@@ -3928,16 +4099,16 @@
         <v>52</v>
       </c>
       <c r="O15" t="s">
-        <v>53</v>
+        <v>220</v>
       </c>
       <c r="P15" t="s">
-        <v>217</v>
+        <v>221</v>
       </c>
       <c r="Q15" t="s">
-        <v>218</v>
+        <v>222</v>
       </c>
       <c r="R15" t="s">
-        <v>219</v>
+        <v>223</v>
       </c>
       <c r="S15" t="s">
         <v>44</v>
@@ -3970,7 +4141,7 @@
         <v>58</v>
       </c>
       <c r="AC15" t="s">
-        <v>61</v>
+        <v>224</v>
       </c>
       <c r="AD15" t="s">
         <v>62</v>
@@ -3979,16 +4150,16 @@
         <v>63</v>
       </c>
       <c r="AF15" t="s">
-        <v>126</v>
+        <v>102</v>
       </c>
       <c r="AG15" t="s">
-        <v>127</v>
+        <v>103</v>
       </c>
       <c r="AH15" t="s">
-        <v>220</v>
+        <v>213</v>
       </c>
       <c r="AI15" t="s">
-        <v>221</v>
+        <v>214</v>
       </c>
       <c r="AJ15" t="s">
         <v>44</v>
@@ -4000,7 +4171,7 @@
         <v>44</v>
       </c>
       <c r="AM15" t="s">
-        <v>44</v>
+        <v>225</v>
       </c>
     </row>
     <row r="16" spans="1:39" x14ac:dyDescent="0.3">
@@ -4008,7 +4179,7 @@
         <v>39</v>
       </c>
       <c r="B16" t="s">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="C16" t="s">
         <v>41</v>
@@ -4023,22 +4194,22 @@
         <v>44</v>
       </c>
       <c r="G16" t="s">
-        <v>69</v>
+        <v>77</v>
       </c>
       <c r="H16" t="s">
-        <v>223</v>
+        <v>227</v>
       </c>
       <c r="I16" t="s">
-        <v>224</v>
+        <v>176</v>
       </c>
       <c r="J16" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
       <c r="K16" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
       <c r="L16" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
       <c r="M16" t="s">
         <v>51</v>
@@ -4050,64 +4221,64 @@
         <v>53</v>
       </c>
       <c r="P16" t="s">
-        <v>228</v>
+        <v>44</v>
       </c>
       <c r="Q16" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="R16" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="S16" t="s">
         <v>44</v>
       </c>
       <c r="T16" t="s">
-        <v>56</v>
+        <v>165</v>
       </c>
       <c r="U16" t="s">
-        <v>56</v>
+        <v>165</v>
       </c>
       <c r="V16" t="s">
         <v>57</v>
       </c>
       <c r="W16" t="s">
-        <v>58</v>
+        <v>166</v>
       </c>
       <c r="X16" t="s">
-        <v>59</v>
+        <v>183</v>
       </c>
       <c r="Y16" t="s">
         <v>60</v>
       </c>
       <c r="Z16" t="s">
-        <v>42</v>
+        <v>183</v>
       </c>
       <c r="AA16" t="s">
-        <v>42</v>
+        <v>184</v>
       </c>
       <c r="AB16" t="s">
-        <v>58</v>
+        <v>185</v>
       </c>
       <c r="AC16" t="s">
-        <v>61</v>
+        <v>186</v>
       </c>
       <c r="AD16" t="s">
-        <v>62</v>
+        <v>233</v>
       </c>
       <c r="AE16" t="s">
         <v>63</v>
       </c>
       <c r="AF16" t="s">
-        <v>64</v>
+        <v>93</v>
       </c>
       <c r="AG16" t="s">
-        <v>65</v>
+        <v>234</v>
       </c>
       <c r="AH16" t="s">
-        <v>231</v>
+        <v>235</v>
       </c>
       <c r="AI16" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="AJ16" t="s">
         <v>44</v>
@@ -4127,13 +4298,13 @@
         <v>39</v>
       </c>
       <c r="B17" t="s">
-        <v>233</v>
+        <v>237</v>
       </c>
       <c r="C17" t="s">
         <v>41</v>
       </c>
       <c r="D17" t="s">
-        <v>234</v>
+        <v>42</v>
       </c>
       <c r="E17" t="s">
         <v>43</v>
@@ -4142,22 +4313,22 @@
         <v>44</v>
       </c>
       <c r="G17" t="s">
-        <v>45</v>
+        <v>77</v>
       </c>
       <c r="H17" t="s">
-        <v>235</v>
+        <v>202</v>
       </c>
       <c r="I17" t="s">
-        <v>47</v>
+        <v>119</v>
       </c>
       <c r="J17" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="K17" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="L17" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="M17" t="s">
         <v>51</v>
@@ -4169,64 +4340,64 @@
         <v>53</v>
       </c>
       <c r="P17" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="Q17" t="s">
-        <v>239</v>
+        <v>242</v>
       </c>
       <c r="R17" t="s">
-        <v>240</v>
+        <v>243</v>
       </c>
       <c r="S17" t="s">
         <v>44</v>
       </c>
       <c r="T17" t="s">
-        <v>84</v>
+        <v>56</v>
       </c>
       <c r="U17" t="s">
-        <v>84</v>
+        <v>56</v>
       </c>
       <c r="V17" t="s">
         <v>57</v>
       </c>
       <c r="W17" t="s">
-        <v>85</v>
+        <v>58</v>
       </c>
       <c r="X17" t="s">
-        <v>241</v>
+        <v>59</v>
       </c>
       <c r="Y17" t="s">
         <v>60</v>
       </c>
       <c r="Z17" t="s">
-        <v>242</v>
+        <v>42</v>
       </c>
       <c r="AA17" t="s">
-        <v>243</v>
+        <v>42</v>
       </c>
       <c r="AB17" t="s">
-        <v>244</v>
+        <v>58</v>
       </c>
       <c r="AC17" t="s">
-        <v>245</v>
+        <v>61</v>
       </c>
       <c r="AD17" t="s">
-        <v>246</v>
+        <v>62</v>
       </c>
       <c r="AE17" t="s">
         <v>63</v>
       </c>
       <c r="AF17" t="s">
-        <v>64</v>
+        <v>126</v>
       </c>
       <c r="AG17" t="s">
-        <v>247</v>
+        <v>127</v>
       </c>
       <c r="AH17" t="s">
-        <v>248</v>
+        <v>244</v>
       </c>
       <c r="AI17" t="s">
-        <v>249</v>
+        <v>245</v>
       </c>
       <c r="AJ17" t="s">
         <v>44</v>
@@ -4238,7 +4409,7 @@
         <v>44</v>
       </c>
       <c r="AM17" t="s">
-        <v>250</v>
+        <v>44</v>
       </c>
     </row>
     <row r="18" spans="1:39" x14ac:dyDescent="0.3">
@@ -4246,13 +4417,13 @@
         <v>39</v>
       </c>
       <c r="B18" t="s">
-        <v>251</v>
+        <v>246</v>
       </c>
       <c r="C18" t="s">
-        <v>130</v>
+        <v>41</v>
       </c>
       <c r="D18" t="s">
-        <v>252</v>
+        <v>42</v>
       </c>
       <c r="E18" t="s">
         <v>43</v>
@@ -4264,88 +4435,88 @@
         <v>69</v>
       </c>
       <c r="H18" t="s">
-        <v>253</v>
+        <v>247</v>
       </c>
       <c r="I18" t="s">
-        <v>44</v>
+        <v>248</v>
       </c>
       <c r="J18" t="s">
-        <v>254</v>
+        <v>249</v>
       </c>
       <c r="K18" t="s">
-        <v>255</v>
+        <v>250</v>
       </c>
       <c r="L18" t="s">
-        <v>256</v>
+        <v>251</v>
       </c>
       <c r="M18" t="s">
         <v>51</v>
       </c>
       <c r="N18" t="s">
-        <v>195</v>
+        <v>52</v>
       </c>
       <c r="O18" t="s">
-        <v>196</v>
+        <v>53</v>
       </c>
       <c r="P18" t="s">
-        <v>44</v>
+        <v>252</v>
       </c>
       <c r="Q18" t="s">
-        <v>257</v>
+        <v>253</v>
       </c>
       <c r="R18" t="s">
-        <v>258</v>
+        <v>254</v>
       </c>
       <c r="S18" t="s">
         <v>44</v>
       </c>
       <c r="T18" t="s">
-        <v>165</v>
+        <v>56</v>
       </c>
       <c r="U18" t="s">
-        <v>165</v>
+        <v>56</v>
       </c>
       <c r="V18" t="s">
         <v>57</v>
       </c>
       <c r="W18" t="s">
-        <v>166</v>
+        <v>58</v>
       </c>
       <c r="X18" t="s">
-        <v>182</v>
+        <v>59</v>
       </c>
       <c r="Y18" t="s">
-        <v>87</v>
+        <v>60</v>
       </c>
       <c r="Z18" t="s">
-        <v>183</v>
+        <v>42</v>
       </c>
       <c r="AA18" t="s">
-        <v>184</v>
+        <v>42</v>
       </c>
       <c r="AB18" t="s">
-        <v>185</v>
+        <v>58</v>
       </c>
       <c r="AC18" t="s">
-        <v>185</v>
+        <v>61</v>
       </c>
       <c r="AD18" t="s">
-        <v>187</v>
+        <v>62</v>
       </c>
       <c r="AE18" t="s">
-        <v>44</v>
+        <v>63</v>
       </c>
       <c r="AF18" t="s">
-        <v>220</v>
+        <v>64</v>
       </c>
       <c r="AG18" t="s">
-        <v>259</v>
+        <v>65</v>
       </c>
       <c r="AH18" t="s">
-        <v>260</v>
+        <v>255</v>
       </c>
       <c r="AI18" t="s">
-        <v>261</v>
+        <v>256</v>
       </c>
       <c r="AJ18" t="s">
         <v>44</v>
@@ -4357,7 +4528,7 @@
         <v>44</v>
       </c>
       <c r="AM18" t="s">
-        <v>262</v>
+        <v>44</v>
       </c>
     </row>
     <row r="19" spans="1:39" x14ac:dyDescent="0.3">
@@ -4365,13 +4536,13 @@
         <v>39</v>
       </c>
       <c r="B19" t="s">
-        <v>263</v>
+        <v>257</v>
       </c>
       <c r="C19" t="s">
         <v>41</v>
       </c>
       <c r="D19" t="s">
-        <v>42</v>
+        <v>258</v>
       </c>
       <c r="E19" t="s">
         <v>43</v>
@@ -4380,22 +4551,22 @@
         <v>44</v>
       </c>
       <c r="G19" t="s">
-        <v>69</v>
+        <v>45</v>
       </c>
       <c r="H19" t="s">
-        <v>70</v>
+        <v>259</v>
       </c>
       <c r="I19" t="s">
         <v>47</v>
       </c>
       <c r="J19" t="s">
-        <v>71</v>
+        <v>260</v>
       </c>
       <c r="K19" t="s">
-        <v>72</v>
+        <v>261</v>
       </c>
       <c r="L19" t="s">
-        <v>73</v>
+        <v>262</v>
       </c>
       <c r="M19" t="s">
         <v>51</v>
@@ -4407,46 +4578,46 @@
         <v>53</v>
       </c>
       <c r="P19" t="s">
-        <v>74</v>
+        <v>263</v>
       </c>
       <c r="Q19" t="s">
-        <v>74</v>
+        <v>263</v>
       </c>
       <c r="R19" t="s">
-        <v>75</v>
+        <v>264</v>
       </c>
       <c r="S19" t="s">
-        <v>264</v>
+        <v>44</v>
       </c>
       <c r="T19" t="s">
-        <v>265</v>
+        <v>84</v>
       </c>
       <c r="U19" t="s">
-        <v>266</v>
+        <v>84</v>
       </c>
       <c r="V19" t="s">
         <v>57</v>
       </c>
       <c r="W19" t="s">
+        <v>85</v>
+      </c>
+      <c r="X19" t="s">
+        <v>265</v>
+      </c>
+      <c r="Y19" t="s">
+        <v>60</v>
+      </c>
+      <c r="Z19" t="s">
+        <v>266</v>
+      </c>
+      <c r="AA19" t="s">
         <v>267</v>
       </c>
-      <c r="X19" t="s">
+      <c r="AB19" t="s">
         <v>268</v>
       </c>
-      <c r="Y19" t="s">
+      <c r="AC19" t="s">
         <v>269</v>
-      </c>
-      <c r="Z19" t="s">
-        <v>42</v>
-      </c>
-      <c r="AA19" t="s">
-        <v>42</v>
-      </c>
-      <c r="AB19" t="s">
-        <v>267</v>
-      </c>
-      <c r="AC19" t="s">
-        <v>267</v>
       </c>
       <c r="AD19" t="s">
         <v>270</v>
@@ -4461,22 +4632,22 @@
         <v>271</v>
       </c>
       <c r="AH19" t="s">
-        <v>66</v>
+        <v>272</v>
       </c>
       <c r="AI19" t="s">
-        <v>67</v>
+        <v>273</v>
       </c>
       <c r="AJ19" t="s">
         <v>44</v>
       </c>
       <c r="AK19" t="s">
-        <v>272</v>
+        <v>44</v>
       </c>
       <c r="AL19" t="s">
-        <v>273</v>
+        <v>44</v>
       </c>
       <c r="AM19" t="s">
-        <v>44</v>
+        <v>274</v>
       </c>
     </row>
     <row r="20" spans="1:39" x14ac:dyDescent="0.3">
@@ -4484,13 +4655,13 @@
         <v>39</v>
       </c>
       <c r="B20" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
       <c r="C20" t="s">
-        <v>41</v>
+        <v>130</v>
       </c>
       <c r="D20" t="s">
-        <v>42</v>
+        <v>276</v>
       </c>
       <c r="E20" t="s">
         <v>43</v>
@@ -4502,100 +4673,100 @@
         <v>69</v>
       </c>
       <c r="H20" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
       <c r="I20" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="J20" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="K20" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="L20" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
       <c r="M20" t="s">
         <v>51</v>
       </c>
       <c r="N20" t="s">
-        <v>52</v>
+        <v>195</v>
       </c>
       <c r="O20" t="s">
-        <v>53</v>
+        <v>196</v>
       </c>
       <c r="P20" t="s">
-        <v>279</v>
+        <v>44</v>
       </c>
       <c r="Q20" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
       <c r="R20" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="S20" t="s">
-        <v>264</v>
+        <v>44</v>
       </c>
       <c r="T20" t="s">
-        <v>281</v>
+        <v>165</v>
       </c>
       <c r="U20" t="s">
-        <v>282</v>
+        <v>165</v>
       </c>
       <c r="V20" t="s">
         <v>57</v>
       </c>
       <c r="W20" t="s">
+        <v>166</v>
+      </c>
+      <c r="X20" t="s">
+        <v>182</v>
+      </c>
+      <c r="Y20" t="s">
+        <v>87</v>
+      </c>
+      <c r="Z20" t="s">
+        <v>183</v>
+      </c>
+      <c r="AA20" t="s">
+        <v>184</v>
+      </c>
+      <c r="AB20" t="s">
+        <v>185</v>
+      </c>
+      <c r="AC20" t="s">
+        <v>185</v>
+      </c>
+      <c r="AD20" t="s">
+        <v>187</v>
+      </c>
+      <c r="AE20" t="s">
+        <v>44</v>
+      </c>
+      <c r="AF20" t="s">
+        <v>244</v>
+      </c>
+      <c r="AG20" t="s">
         <v>283</v>
       </c>
-      <c r="X20" t="s">
-        <v>268</v>
-      </c>
-      <c r="Y20" t="s">
+      <c r="AH20" t="s">
         <v>284</v>
       </c>
-      <c r="Z20" t="s">
+      <c r="AI20" t="s">
         <v>285</v>
       </c>
-      <c r="AA20" t="s">
-        <v>189</v>
-      </c>
-      <c r="AB20" t="s">
+      <c r="AJ20" t="s">
+        <v>44</v>
+      </c>
+      <c r="AK20" t="s">
+        <v>44</v>
+      </c>
+      <c r="AL20" t="s">
+        <v>44</v>
+      </c>
+      <c r="AM20" t="s">
         <v>286</v>
-      </c>
-      <c r="AC20" t="s">
-        <v>286</v>
-      </c>
-      <c r="AD20" t="s">
-        <v>287</v>
-      </c>
-      <c r="AE20" t="s">
-        <v>63</v>
-      </c>
-      <c r="AF20" t="s">
-        <v>64</v>
-      </c>
-      <c r="AG20" t="s">
-        <v>288</v>
-      </c>
-      <c r="AH20" t="s">
-        <v>66</v>
-      </c>
-      <c r="AI20" t="s">
-        <v>67</v>
-      </c>
-      <c r="AJ20" t="s">
-        <v>44</v>
-      </c>
-      <c r="AK20" t="s">
-        <v>272</v>
-      </c>
-      <c r="AL20" t="s">
-        <v>273</v>
-      </c>
-      <c r="AM20" t="s">
-        <v>44</v>
       </c>
     </row>
     <row r="21" spans="1:39" x14ac:dyDescent="0.3">
@@ -4603,7 +4774,7 @@
         <v>39</v>
       </c>
       <c r="B21" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="C21" t="s">
         <v>41</v>
@@ -4618,22 +4789,22 @@
         <v>44</v>
       </c>
       <c r="G21" t="s">
-        <v>290</v>
+        <v>69</v>
       </c>
       <c r="H21" t="s">
-        <v>291</v>
+        <v>70</v>
       </c>
       <c r="I21" t="s">
-        <v>224</v>
+        <v>47</v>
       </c>
       <c r="J21" t="s">
-        <v>292</v>
+        <v>71</v>
       </c>
       <c r="K21" t="s">
-        <v>293</v>
+        <v>72</v>
       </c>
       <c r="L21" t="s">
-        <v>294</v>
+        <v>73</v>
       </c>
       <c r="M21" t="s">
         <v>51</v>
@@ -4642,37 +4813,37 @@
         <v>52</v>
       </c>
       <c r="O21" t="s">
-        <v>295</v>
+        <v>53</v>
       </c>
       <c r="P21" t="s">
-        <v>44</v>
+        <v>74</v>
       </c>
       <c r="Q21" t="s">
-        <v>296</v>
+        <v>74</v>
       </c>
       <c r="R21" t="s">
-        <v>297</v>
+        <v>75</v>
       </c>
       <c r="S21" t="s">
-        <v>264</v>
+        <v>288</v>
       </c>
       <c r="T21" t="s">
-        <v>298</v>
+        <v>289</v>
       </c>
       <c r="U21" t="s">
-        <v>299</v>
+        <v>290</v>
       </c>
       <c r="V21" t="s">
         <v>57</v>
       </c>
       <c r="W21" t="s">
-        <v>300</v>
+        <v>291</v>
       </c>
       <c r="X21" t="s">
-        <v>301</v>
+        <v>292</v>
       </c>
       <c r="Y21" t="s">
-        <v>60</v>
+        <v>293</v>
       </c>
       <c r="Z21" t="s">
         <v>42</v>
@@ -4681,13 +4852,13 @@
         <v>42</v>
       </c>
       <c r="AB21" t="s">
-        <v>300</v>
+        <v>291</v>
       </c>
       <c r="AC21" t="s">
-        <v>300</v>
+        <v>291</v>
       </c>
       <c r="AD21" t="s">
-        <v>302</v>
+        <v>294</v>
       </c>
       <c r="AE21" t="s">
         <v>63</v>
@@ -4696,22 +4867,22 @@
         <v>64</v>
       </c>
       <c r="AG21" t="s">
-        <v>303</v>
+        <v>295</v>
       </c>
       <c r="AH21" t="s">
-        <v>137</v>
+        <v>66</v>
       </c>
       <c r="AI21" t="s">
-        <v>138</v>
+        <v>67</v>
       </c>
       <c r="AJ21" t="s">
         <v>44</v>
       </c>
       <c r="AK21" t="s">
-        <v>272</v>
+        <v>296</v>
       </c>
       <c r="AL21" t="s">
-        <v>273</v>
+        <v>297</v>
       </c>
       <c r="AM21" t="s">
         <v>44</v>
@@ -4722,7 +4893,7 @@
         <v>39</v>
       </c>
       <c r="B22" t="s">
-        <v>304</v>
+        <v>298</v>
       </c>
       <c r="C22" t="s">
         <v>41</v>
@@ -4731,28 +4902,28 @@
         <v>42</v>
       </c>
       <c r="E22" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="F22" t="s">
         <v>44</v>
       </c>
       <c r="G22" t="s">
-        <v>44</v>
+        <v>69</v>
       </c>
       <c r="H22" t="s">
-        <v>305</v>
+        <v>299</v>
       </c>
       <c r="I22" t="s">
-        <v>224</v>
+        <v>47</v>
       </c>
       <c r="J22" t="s">
-        <v>306</v>
+        <v>300</v>
       </c>
       <c r="K22" t="s">
-        <v>307</v>
+        <v>301</v>
       </c>
       <c r="L22" t="s">
-        <v>308</v>
+        <v>302</v>
       </c>
       <c r="M22" t="s">
         <v>51</v>
@@ -4761,76 +4932,76 @@
         <v>52</v>
       </c>
       <c r="O22" t="s">
-        <v>309</v>
+        <v>53</v>
       </c>
       <c r="P22" t="s">
-        <v>310</v>
+        <v>303</v>
       </c>
       <c r="Q22" t="s">
-        <v>311</v>
+        <v>303</v>
       </c>
       <c r="R22" t="s">
-        <v>312</v>
+        <v>304</v>
       </c>
       <c r="S22" t="s">
-        <v>264</v>
+        <v>288</v>
       </c>
       <c r="T22" t="s">
-        <v>298</v>
+        <v>305</v>
       </c>
       <c r="U22" t="s">
-        <v>299</v>
+        <v>306</v>
       </c>
       <c r="V22" t="s">
         <v>57</v>
       </c>
       <c r="W22" t="s">
-        <v>300</v>
+        <v>307</v>
       </c>
       <c r="X22" t="s">
-        <v>42</v>
+        <v>292</v>
       </c>
       <c r="Y22" t="s">
-        <v>42</v>
+        <v>308</v>
       </c>
       <c r="Z22" t="s">
-        <v>313</v>
+        <v>309</v>
       </c>
       <c r="AA22" t="s">
-        <v>314</v>
+        <v>189</v>
       </c>
       <c r="AB22" t="s">
-        <v>315</v>
+        <v>310</v>
       </c>
       <c r="AC22" t="s">
-        <v>315</v>
+        <v>310</v>
       </c>
       <c r="AD22" t="s">
-        <v>315</v>
+        <v>311</v>
       </c>
       <c r="AE22" t="s">
         <v>63</v>
       </c>
       <c r="AF22" t="s">
-        <v>316</v>
+        <v>64</v>
       </c>
       <c r="AG22" t="s">
-        <v>315</v>
+        <v>312</v>
       </c>
       <c r="AH22" t="s">
-        <v>184</v>
+        <v>66</v>
       </c>
       <c r="AI22" t="s">
-        <v>317</v>
+        <v>67</v>
       </c>
       <c r="AJ22" t="s">
         <v>44</v>
       </c>
       <c r="AK22" t="s">
-        <v>272</v>
+        <v>296</v>
       </c>
       <c r="AL22" t="s">
-        <v>273</v>
+        <v>297</v>
       </c>
       <c r="AM22" t="s">
         <v>44</v>
@@ -4841,7 +5012,7 @@
         <v>39</v>
       </c>
       <c r="B23" t="s">
-        <v>318</v>
+        <v>313</v>
       </c>
       <c r="C23" t="s">
         <v>41</v>
@@ -4856,100 +5027,100 @@
         <v>44</v>
       </c>
       <c r="G23" t="s">
-        <v>69</v>
+        <v>314</v>
       </c>
       <c r="H23" t="s">
-        <v>107</v>
+        <v>315</v>
       </c>
       <c r="I23" t="s">
-        <v>141</v>
+        <v>248</v>
       </c>
       <c r="J23" t="s">
-        <v>319</v>
+        <v>316</v>
       </c>
       <c r="K23" t="s">
-        <v>320</v>
+        <v>317</v>
       </c>
       <c r="L23" t="s">
-        <v>321</v>
+        <v>318</v>
       </c>
       <c r="M23" t="s">
         <v>51</v>
       </c>
       <c r="N23" t="s">
-        <v>195</v>
+        <v>52</v>
       </c>
       <c r="O23" t="s">
-        <v>196</v>
+        <v>319</v>
       </c>
       <c r="P23" t="s">
+        <v>44</v>
+      </c>
+      <c r="Q23" t="s">
+        <v>320</v>
+      </c>
+      <c r="R23" t="s">
+        <v>321</v>
+      </c>
+      <c r="S23" t="s">
+        <v>288</v>
+      </c>
+      <c r="T23" t="s">
         <v>322</v>
       </c>
-      <c r="Q23" t="s">
-        <v>322</v>
-      </c>
-      <c r="R23" t="s">
+      <c r="U23" t="s">
         <v>323</v>
-      </c>
-      <c r="S23" t="s">
-        <v>264</v>
-      </c>
-      <c r="T23" t="s">
-        <v>281</v>
-      </c>
-      <c r="U23" t="s">
-        <v>282</v>
       </c>
       <c r="V23" t="s">
         <v>57</v>
       </c>
       <c r="W23" t="s">
-        <v>283</v>
+        <v>324</v>
       </c>
       <c r="X23" t="s">
-        <v>268</v>
+        <v>325</v>
       </c>
       <c r="Y23" t="s">
-        <v>284</v>
+        <v>60</v>
       </c>
       <c r="Z23" t="s">
-        <v>285</v>
+        <v>42</v>
       </c>
       <c r="AA23" t="s">
-        <v>189</v>
+        <v>42</v>
       </c>
       <c r="AB23" t="s">
-        <v>286</v>
+        <v>324</v>
       </c>
       <c r="AC23" t="s">
-        <v>286</v>
+        <v>324</v>
       </c>
       <c r="AD23" t="s">
-        <v>287</v>
+        <v>326</v>
       </c>
       <c r="AE23" t="s">
         <v>63</v>
       </c>
       <c r="AF23" t="s">
-        <v>102</v>
+        <v>64</v>
       </c>
       <c r="AG23" t="s">
-        <v>324</v>
+        <v>327</v>
       </c>
       <c r="AH23" t="s">
-        <v>89</v>
+        <v>137</v>
       </c>
       <c r="AI23" t="s">
-        <v>147</v>
+        <v>138</v>
       </c>
       <c r="AJ23" t="s">
         <v>44</v>
       </c>
       <c r="AK23" t="s">
-        <v>272</v>
+        <v>296</v>
       </c>
       <c r="AL23" t="s">
-        <v>273</v>
+        <v>297</v>
       </c>
       <c r="AM23" t="s">
         <v>44</v>
@@ -4960,7 +5131,7 @@
         <v>39</v>
       </c>
       <c r="B24" t="s">
-        <v>325</v>
+        <v>328</v>
       </c>
       <c r="C24" t="s">
         <v>41</v>
@@ -4978,19 +5149,19 @@
         <v>44</v>
       </c>
       <c r="H24" t="s">
-        <v>305</v>
+        <v>329</v>
       </c>
       <c r="I24" t="s">
-        <v>224</v>
+        <v>248</v>
       </c>
       <c r="J24" t="s">
-        <v>326</v>
+        <v>330</v>
       </c>
       <c r="K24" t="s">
-        <v>327</v>
+        <v>331</v>
       </c>
       <c r="L24" t="s">
-        <v>328</v>
+        <v>332</v>
       </c>
       <c r="M24" t="s">
         <v>51</v>
@@ -4999,31 +5170,31 @@
         <v>52</v>
       </c>
       <c r="O24" t="s">
-        <v>123</v>
+        <v>333</v>
       </c>
       <c r="P24" t="s">
-        <v>329</v>
+        <v>334</v>
       </c>
       <c r="Q24" t="s">
-        <v>329</v>
+        <v>335</v>
       </c>
       <c r="R24" t="s">
-        <v>330</v>
+        <v>336</v>
       </c>
       <c r="S24" t="s">
-        <v>264</v>
+        <v>288</v>
       </c>
       <c r="T24" t="s">
-        <v>281</v>
+        <v>322</v>
       </c>
       <c r="U24" t="s">
-        <v>282</v>
+        <v>323</v>
       </c>
       <c r="V24" t="s">
         <v>57</v>
       </c>
       <c r="W24" t="s">
-        <v>283</v>
+        <v>324</v>
       </c>
       <c r="X24" t="s">
         <v>42</v>
@@ -5032,43 +5203,43 @@
         <v>42</v>
       </c>
       <c r="Z24" t="s">
-        <v>331</v>
+        <v>337</v>
       </c>
       <c r="AA24" t="s">
-        <v>332</v>
+        <v>338</v>
       </c>
       <c r="AB24" t="s">
-        <v>333</v>
+        <v>339</v>
       </c>
       <c r="AC24" t="s">
-        <v>333</v>
+        <v>339</v>
       </c>
       <c r="AD24" t="s">
-        <v>333</v>
+        <v>339</v>
       </c>
       <c r="AE24" t="s">
         <v>63</v>
       </c>
       <c r="AF24" t="s">
-        <v>316</v>
+        <v>340</v>
       </c>
       <c r="AG24" t="s">
-        <v>333</v>
+        <v>339</v>
       </c>
       <c r="AH24" t="s">
         <v>184</v>
       </c>
       <c r="AI24" t="s">
-        <v>317</v>
+        <v>341</v>
       </c>
       <c r="AJ24" t="s">
-        <v>334</v>
+        <v>44</v>
       </c>
       <c r="AK24" t="s">
-        <v>335</v>
+        <v>296</v>
       </c>
       <c r="AL24" t="s">
-        <v>336</v>
+        <v>297</v>
       </c>
       <c r="AM24" t="s">
         <v>44</v>
@@ -5079,7 +5250,7 @@
         <v>39</v>
       </c>
       <c r="B25" t="s">
-        <v>337</v>
+        <v>342</v>
       </c>
       <c r="C25" t="s">
         <v>41</v>
@@ -5088,91 +5259,91 @@
         <v>42</v>
       </c>
       <c r="E25" t="s">
-        <v>338</v>
+        <v>43</v>
       </c>
       <c r="F25" t="s">
-        <v>338</v>
+        <v>44</v>
       </c>
       <c r="G25" t="s">
-        <v>339</v>
+        <v>69</v>
       </c>
       <c r="H25" t="s">
-        <v>340</v>
+        <v>107</v>
       </c>
       <c r="I25" t="s">
-        <v>341</v>
+        <v>141</v>
       </c>
       <c r="J25" t="s">
-        <v>342</v>
+        <v>343</v>
       </c>
       <c r="K25" t="s">
-        <v>343</v>
+        <v>344</v>
       </c>
       <c r="L25" t="s">
-        <v>344</v>
+        <v>345</v>
       </c>
       <c r="M25" t="s">
         <v>51</v>
       </c>
       <c r="N25" t="s">
-        <v>52</v>
+        <v>195</v>
       </c>
       <c r="O25" t="s">
-        <v>53</v>
+        <v>196</v>
       </c>
       <c r="P25" t="s">
-        <v>44</v>
+        <v>346</v>
       </c>
       <c r="Q25" t="s">
-        <v>345</v>
+        <v>346</v>
       </c>
       <c r="R25" t="s">
-        <v>346</v>
+        <v>347</v>
       </c>
       <c r="S25" t="s">
-        <v>264</v>
+        <v>288</v>
       </c>
       <c r="T25" t="s">
-        <v>281</v>
+        <v>305</v>
       </c>
       <c r="U25" t="s">
-        <v>282</v>
+        <v>306</v>
       </c>
       <c r="V25" t="s">
         <v>57</v>
       </c>
       <c r="W25" t="s">
-        <v>283</v>
+        <v>307</v>
       </c>
       <c r="X25" t="s">
-        <v>347</v>
+        <v>292</v>
       </c>
       <c r="Y25" t="s">
-        <v>348</v>
+        <v>308</v>
       </c>
       <c r="Z25" t="s">
-        <v>349</v>
+        <v>309</v>
       </c>
       <c r="AA25" t="s">
-        <v>184</v>
+        <v>189</v>
       </c>
       <c r="AB25" t="s">
-        <v>350</v>
+        <v>310</v>
       </c>
       <c r="AC25" t="s">
-        <v>350</v>
+        <v>310</v>
       </c>
       <c r="AD25" t="s">
-        <v>351</v>
+        <v>311</v>
       </c>
       <c r="AE25" t="s">
         <v>63</v>
       </c>
       <c r="AF25" t="s">
-        <v>199</v>
+        <v>102</v>
       </c>
       <c r="AG25" t="s">
-        <v>352</v>
+        <v>348</v>
       </c>
       <c r="AH25" t="s">
         <v>89</v>
@@ -5181,13 +5352,13 @@
         <v>147</v>
       </c>
       <c r="AJ25" t="s">
-        <v>334</v>
+        <v>44</v>
       </c>
       <c r="AK25" t="s">
-        <v>353</v>
+        <v>296</v>
       </c>
       <c r="AL25" t="s">
-        <v>354</v>
+        <v>297</v>
       </c>
       <c r="AM25" t="s">
         <v>44</v>
@@ -5198,13 +5369,13 @@
         <v>39</v>
       </c>
       <c r="B26" t="s">
-        <v>355</v>
+        <v>349</v>
       </c>
       <c r="C26" t="s">
-        <v>41</v>
+        <v>130</v>
       </c>
       <c r="D26" t="s">
-        <v>42</v>
+        <v>350</v>
       </c>
       <c r="E26" t="s">
         <v>43</v>
@@ -5216,100 +5387,100 @@
         <v>69</v>
       </c>
       <c r="H26" t="s">
-        <v>356</v>
+        <v>299</v>
       </c>
       <c r="I26" t="s">
-        <v>141</v>
+        <v>44</v>
       </c>
       <c r="J26" t="s">
-        <v>357</v>
+        <v>351</v>
       </c>
       <c r="K26" t="s">
-        <v>358</v>
+        <v>352</v>
       </c>
       <c r="L26" t="s">
-        <v>359</v>
+        <v>353</v>
       </c>
       <c r="M26" t="s">
         <v>51</v>
       </c>
       <c r="N26" t="s">
-        <v>195</v>
+        <v>52</v>
       </c>
       <c r="O26" t="s">
-        <v>196</v>
+        <v>53</v>
       </c>
       <c r="P26" t="s">
-        <v>360</v>
+        <v>44</v>
       </c>
       <c r="Q26" t="s">
-        <v>360</v>
+        <v>354</v>
       </c>
       <c r="R26" t="s">
-        <v>361</v>
+        <v>355</v>
       </c>
       <c r="S26" t="s">
-        <v>264</v>
+        <v>288</v>
       </c>
       <c r="T26" t="s">
-        <v>265</v>
+        <v>305</v>
       </c>
       <c r="U26" t="s">
-        <v>266</v>
+        <v>306</v>
       </c>
       <c r="V26" t="s">
         <v>57</v>
       </c>
       <c r="W26" t="s">
-        <v>267</v>
+        <v>307</v>
       </c>
       <c r="X26" t="s">
-        <v>362</v>
+        <v>292</v>
       </c>
       <c r="Y26" t="s">
-        <v>87</v>
+        <v>308</v>
       </c>
       <c r="Z26" t="s">
-        <v>363</v>
+        <v>309</v>
       </c>
       <c r="AA26" t="s">
-        <v>184</v>
+        <v>189</v>
       </c>
       <c r="AB26" t="s">
-        <v>364</v>
+        <v>310</v>
       </c>
       <c r="AC26" t="s">
-        <v>364</v>
+        <v>310</v>
       </c>
       <c r="AD26" t="s">
-        <v>365</v>
+        <v>311</v>
       </c>
       <c r="AE26" t="s">
         <v>63</v>
       </c>
       <c r="AF26" t="s">
-        <v>102</v>
+        <v>356</v>
       </c>
       <c r="AG26" t="s">
-        <v>366</v>
+        <v>357</v>
       </c>
       <c r="AH26" t="s">
-        <v>367</v>
+        <v>358</v>
       </c>
       <c r="AI26" t="s">
-        <v>368</v>
+        <v>359</v>
       </c>
       <c r="AJ26" t="s">
-        <v>334</v>
+        <v>360</v>
       </c>
       <c r="AK26" t="s">
-        <v>369</v>
+        <v>361</v>
       </c>
       <c r="AL26" t="s">
-        <v>370</v>
+        <v>362</v>
       </c>
       <c r="AM26" t="s">
-        <v>44</v>
+        <v>363</v>
       </c>
     </row>
     <row r="27" spans="1:39" x14ac:dyDescent="0.3">
@@ -5317,7 +5488,7 @@
         <v>39</v>
       </c>
       <c r="B27" t="s">
-        <v>371</v>
+        <v>364</v>
       </c>
       <c r="C27" t="s">
         <v>41</v>
@@ -5326,28 +5497,28 @@
         <v>42</v>
       </c>
       <c r="E27" t="s">
-        <v>372</v>
+        <v>44</v>
       </c>
       <c r="F27" t="s">
         <v>44</v>
       </c>
       <c r="G27" t="s">
-        <v>373</v>
+        <v>44</v>
       </c>
       <c r="H27" t="s">
-        <v>374</v>
+        <v>329</v>
       </c>
       <c r="I27" t="s">
-        <v>141</v>
+        <v>248</v>
       </c>
       <c r="J27" t="s">
-        <v>375</v>
+        <v>365</v>
       </c>
       <c r="K27" t="s">
-        <v>376</v>
+        <v>366</v>
       </c>
       <c r="L27" t="s">
-        <v>377</v>
+        <v>367</v>
       </c>
       <c r="M27" t="s">
         <v>51</v>
@@ -5356,76 +5527,76 @@
         <v>52</v>
       </c>
       <c r="O27" t="s">
-        <v>378</v>
+        <v>123</v>
       </c>
       <c r="P27" t="s">
-        <v>44</v>
+        <v>368</v>
       </c>
       <c r="Q27" t="s">
-        <v>379</v>
+        <v>368</v>
       </c>
       <c r="R27" t="s">
-        <v>380</v>
+        <v>369</v>
       </c>
       <c r="S27" t="s">
-        <v>264</v>
+        <v>288</v>
       </c>
       <c r="T27" t="s">
-        <v>265</v>
+        <v>305</v>
       </c>
       <c r="U27" t="s">
-        <v>266</v>
+        <v>306</v>
       </c>
       <c r="V27" t="s">
         <v>57</v>
       </c>
       <c r="W27" t="s">
-        <v>267</v>
+        <v>307</v>
       </c>
       <c r="X27" t="s">
-        <v>59</v>
+        <v>42</v>
       </c>
       <c r="Y27" t="s">
-        <v>87</v>
+        <v>42</v>
       </c>
       <c r="Z27" t="s">
-        <v>381</v>
+        <v>370</v>
       </c>
       <c r="AA27" t="s">
-        <v>382</v>
+        <v>371</v>
       </c>
       <c r="AB27" t="s">
-        <v>383</v>
+        <v>210</v>
       </c>
       <c r="AC27" t="s">
-        <v>383</v>
+        <v>210</v>
       </c>
       <c r="AD27" t="s">
-        <v>384</v>
+        <v>210</v>
       </c>
       <c r="AE27" t="s">
         <v>63</v>
       </c>
       <c r="AF27" t="s">
-        <v>385</v>
+        <v>340</v>
       </c>
       <c r="AG27" t="s">
-        <v>386</v>
+        <v>210</v>
       </c>
       <c r="AH27" t="s">
         <v>184</v>
       </c>
       <c r="AI27" t="s">
-        <v>317</v>
+        <v>341</v>
       </c>
       <c r="AJ27" t="s">
-        <v>334</v>
+        <v>360</v>
       </c>
       <c r="AK27" t="s">
-        <v>387</v>
+        <v>372</v>
       </c>
       <c r="AL27" t="s">
-        <v>370</v>
+        <v>362</v>
       </c>
       <c r="AM27" t="s">
         <v>44</v>
@@ -5436,37 +5607,37 @@
         <v>39</v>
       </c>
       <c r="B28" t="s">
-        <v>388</v>
+        <v>373</v>
       </c>
       <c r="C28" t="s">
-        <v>41</v>
+        <v>130</v>
       </c>
       <c r="D28" t="s">
-        <v>42</v>
+        <v>374</v>
       </c>
       <c r="E28" t="s">
-        <v>43</v>
+        <v>375</v>
       </c>
       <c r="F28" t="s">
-        <v>44</v>
+        <v>375</v>
       </c>
       <c r="G28" t="s">
-        <v>45</v>
+        <v>376</v>
       </c>
       <c r="H28" t="s">
-        <v>46</v>
+        <v>377</v>
       </c>
       <c r="I28" t="s">
-        <v>119</v>
+        <v>44</v>
       </c>
       <c r="J28" t="s">
-        <v>389</v>
+        <v>378</v>
       </c>
       <c r="K28" t="s">
-        <v>390</v>
+        <v>379</v>
       </c>
       <c r="L28" t="s">
-        <v>391</v>
+        <v>380</v>
       </c>
       <c r="M28" t="s">
         <v>51</v>
@@ -5475,79 +5646,79 @@
         <v>52</v>
       </c>
       <c r="O28" t="s">
-        <v>392</v>
+        <v>53</v>
       </c>
       <c r="P28" t="s">
         <v>44</v>
       </c>
       <c r="Q28" t="s">
-        <v>393</v>
+        <v>381</v>
       </c>
       <c r="R28" t="s">
-        <v>394</v>
+        <v>382</v>
       </c>
       <c r="S28" t="s">
-        <v>264</v>
+        <v>288</v>
       </c>
       <c r="T28" t="s">
-        <v>298</v>
+        <v>305</v>
       </c>
       <c r="U28" t="s">
-        <v>299</v>
+        <v>306</v>
       </c>
       <c r="V28" t="s">
         <v>57</v>
       </c>
       <c r="W28" t="s">
-        <v>300</v>
+        <v>307</v>
       </c>
       <c r="X28" t="s">
-        <v>395</v>
+        <v>383</v>
       </c>
       <c r="Y28" t="s">
         <v>60</v>
       </c>
       <c r="Z28" t="s">
-        <v>42</v>
+        <v>384</v>
       </c>
       <c r="AA28" t="s">
-        <v>42</v>
+        <v>184</v>
       </c>
       <c r="AB28" t="s">
-        <v>300</v>
+        <v>385</v>
       </c>
       <c r="AC28" t="s">
-        <v>300</v>
+        <v>385</v>
       </c>
       <c r="AD28" t="s">
-        <v>396</v>
+        <v>386</v>
       </c>
       <c r="AE28" t="s">
         <v>63</v>
       </c>
       <c r="AF28" t="s">
-        <v>64</v>
+        <v>102</v>
       </c>
       <c r="AG28" t="s">
-        <v>397</v>
+        <v>387</v>
       </c>
       <c r="AH28" t="s">
-        <v>398</v>
+        <v>104</v>
       </c>
       <c r="AI28" t="s">
-        <v>399</v>
+        <v>128</v>
       </c>
       <c r="AJ28" t="s">
-        <v>334</v>
+        <v>388</v>
       </c>
       <c r="AK28" t="s">
-        <v>400</v>
+        <v>389</v>
       </c>
       <c r="AL28" t="s">
-        <v>401</v>
+        <v>390</v>
       </c>
       <c r="AM28" t="s">
-        <v>44</v>
+        <v>225</v>
       </c>
     </row>
     <row r="29" spans="1:39" x14ac:dyDescent="0.3">
@@ -5555,7 +5726,7 @@
         <v>39</v>
       </c>
       <c r="B29" t="s">
-        <v>402</v>
+        <v>391</v>
       </c>
       <c r="C29" t="s">
         <v>41</v>
@@ -5564,28 +5735,28 @@
         <v>42</v>
       </c>
       <c r="E29" t="s">
-        <v>43</v>
+        <v>375</v>
       </c>
       <c r="F29" t="s">
-        <v>44</v>
+        <v>375</v>
       </c>
       <c r="G29" t="s">
-        <v>290</v>
+        <v>376</v>
       </c>
       <c r="H29" t="s">
-        <v>291</v>
+        <v>377</v>
       </c>
       <c r="I29" t="s">
-        <v>176</v>
+        <v>392</v>
       </c>
       <c r="J29" t="s">
-        <v>403</v>
+        <v>393</v>
       </c>
       <c r="K29" t="s">
-        <v>404</v>
+        <v>394</v>
       </c>
       <c r="L29" t="s">
-        <v>405</v>
+        <v>395</v>
       </c>
       <c r="M29" t="s">
         <v>51</v>
@@ -5600,70 +5771,70 @@
         <v>44</v>
       </c>
       <c r="Q29" t="s">
-        <v>406</v>
+        <v>396</v>
       </c>
       <c r="R29" t="s">
-        <v>407</v>
+        <v>397</v>
       </c>
       <c r="S29" t="s">
-        <v>264</v>
+        <v>288</v>
       </c>
       <c r="T29" t="s">
-        <v>298</v>
+        <v>305</v>
       </c>
       <c r="U29" t="s">
-        <v>299</v>
+        <v>306</v>
       </c>
       <c r="V29" t="s">
         <v>57</v>
       </c>
       <c r="W29" t="s">
-        <v>283</v>
+        <v>307</v>
       </c>
       <c r="X29" t="s">
-        <v>349</v>
+        <v>398</v>
       </c>
       <c r="Y29" t="s">
-        <v>60</v>
+        <v>399</v>
       </c>
       <c r="Z29" t="s">
-        <v>349</v>
+        <v>384</v>
       </c>
       <c r="AA29" t="s">
         <v>184</v>
       </c>
       <c r="AB29" t="s">
-        <v>350</v>
+        <v>385</v>
       </c>
       <c r="AC29" t="s">
-        <v>350</v>
+        <v>385</v>
       </c>
       <c r="AD29" t="s">
-        <v>286</v>
+        <v>400</v>
       </c>
       <c r="AE29" t="s">
         <v>63</v>
       </c>
       <c r="AF29" t="s">
-        <v>102</v>
+        <v>199</v>
       </c>
       <c r="AG29" t="s">
-        <v>408</v>
+        <v>401</v>
       </c>
       <c r="AH29" t="s">
-        <v>398</v>
+        <v>89</v>
       </c>
       <c r="AI29" t="s">
-        <v>409</v>
+        <v>147</v>
       </c>
       <c r="AJ29" t="s">
-        <v>334</v>
+        <v>360</v>
       </c>
       <c r="AK29" t="s">
-        <v>410</v>
+        <v>402</v>
       </c>
       <c r="AL29" t="s">
-        <v>411</v>
+        <v>390</v>
       </c>
       <c r="AM29" t="s">
         <v>44</v>
@@ -5674,7 +5845,7 @@
         <v>39</v>
       </c>
       <c r="B30" t="s">
-        <v>412</v>
+        <v>403</v>
       </c>
       <c r="C30" t="s">
         <v>41</v>
@@ -5683,106 +5854,106 @@
         <v>42</v>
       </c>
       <c r="E30" t="s">
-        <v>338</v>
+        <v>43</v>
       </c>
       <c r="F30" t="s">
-        <v>338</v>
+        <v>44</v>
       </c>
       <c r="G30" t="s">
-        <v>339</v>
+        <v>69</v>
       </c>
       <c r="H30" t="s">
-        <v>340</v>
+        <v>404</v>
       </c>
       <c r="I30" t="s">
-        <v>176</v>
+        <v>141</v>
       </c>
       <c r="J30" t="s">
-        <v>413</v>
+        <v>405</v>
       </c>
       <c r="K30" t="s">
-        <v>414</v>
+        <v>406</v>
       </c>
       <c r="L30" t="s">
-        <v>415</v>
+        <v>407</v>
       </c>
       <c r="M30" t="s">
         <v>51</v>
       </c>
       <c r="N30" t="s">
-        <v>52</v>
+        <v>195</v>
       </c>
       <c r="O30" t="s">
-        <v>53</v>
+        <v>196</v>
       </c>
       <c r="P30" t="s">
-        <v>44</v>
+        <v>408</v>
       </c>
       <c r="Q30" t="s">
-        <v>416</v>
+        <v>408</v>
       </c>
       <c r="R30" t="s">
-        <v>417</v>
+        <v>409</v>
       </c>
       <c r="S30" t="s">
-        <v>264</v>
+        <v>288</v>
       </c>
       <c r="T30" t="s">
-        <v>298</v>
+        <v>289</v>
       </c>
       <c r="U30" t="s">
-        <v>299</v>
+        <v>290</v>
       </c>
       <c r="V30" t="s">
         <v>57</v>
       </c>
       <c r="W30" t="s">
-        <v>283</v>
+        <v>291</v>
       </c>
       <c r="X30" t="s">
-        <v>418</v>
+        <v>410</v>
       </c>
       <c r="Y30" t="s">
-        <v>419</v>
+        <v>87</v>
       </c>
       <c r="Z30" t="s">
-        <v>42</v>
+        <v>411</v>
       </c>
       <c r="AA30" t="s">
-        <v>42</v>
+        <v>184</v>
       </c>
       <c r="AB30" t="s">
-        <v>283</v>
+        <v>412</v>
       </c>
       <c r="AC30" t="s">
-        <v>283</v>
+        <v>412</v>
       </c>
       <c r="AD30" t="s">
-        <v>420</v>
+        <v>413</v>
       </c>
       <c r="AE30" t="s">
         <v>63</v>
       </c>
       <c r="AF30" t="s">
-        <v>385</v>
+        <v>102</v>
       </c>
       <c r="AG30" t="s">
-        <v>421</v>
+        <v>414</v>
       </c>
       <c r="AH30" t="s">
-        <v>316</v>
+        <v>388</v>
       </c>
       <c r="AI30" t="s">
-        <v>422</v>
+        <v>415</v>
       </c>
       <c r="AJ30" t="s">
-        <v>334</v>
+        <v>360</v>
       </c>
       <c r="AK30" t="s">
-        <v>423</v>
+        <v>416</v>
       </c>
       <c r="AL30" t="s">
-        <v>411</v>
+        <v>417</v>
       </c>
       <c r="AM30" t="s">
         <v>44</v>
@@ -5793,37 +5964,37 @@
         <v>39</v>
       </c>
       <c r="B31" t="s">
-        <v>424</v>
+        <v>418</v>
       </c>
       <c r="C31" t="s">
         <v>41</v>
       </c>
       <c r="D31" t="s">
-        <v>425</v>
+        <v>42</v>
       </c>
       <c r="E31" t="s">
-        <v>426</v>
+        <v>419</v>
       </c>
       <c r="F31" t="s">
-        <v>373</v>
+        <v>44</v>
       </c>
       <c r="G31" t="s">
-        <v>427</v>
+        <v>420</v>
       </c>
       <c r="H31" t="s">
-        <v>427</v>
+        <v>421</v>
       </c>
       <c r="I31" t="s">
-        <v>44</v>
+        <v>141</v>
       </c>
       <c r="J31" t="s">
-        <v>428</v>
+        <v>422</v>
       </c>
       <c r="K31" t="s">
-        <v>429</v>
+        <v>423</v>
       </c>
       <c r="L31" t="s">
-        <v>430</v>
+        <v>424</v>
       </c>
       <c r="M31" t="s">
         <v>51</v>
@@ -5832,79 +6003,674 @@
         <v>52</v>
       </c>
       <c r="O31" t="s">
-        <v>431</v>
+        <v>425</v>
       </c>
       <c r="P31" t="s">
         <v>44</v>
       </c>
       <c r="Q31" t="s">
-        <v>432</v>
+        <v>426</v>
       </c>
       <c r="R31" t="s">
-        <v>433</v>
+        <v>427</v>
       </c>
       <c r="S31" t="s">
-        <v>434</v>
+        <v>288</v>
       </c>
       <c r="T31" t="s">
-        <v>435</v>
+        <v>289</v>
       </c>
       <c r="U31" t="s">
-        <v>436</v>
+        <v>290</v>
       </c>
       <c r="V31" t="s">
         <v>57</v>
       </c>
       <c r="W31" t="s">
+        <v>291</v>
+      </c>
+      <c r="X31" t="s">
+        <v>59</v>
+      </c>
+      <c r="Y31" t="s">
+        <v>87</v>
+      </c>
+      <c r="Z31" t="s">
+        <v>428</v>
+      </c>
+      <c r="AA31" t="s">
+        <v>429</v>
+      </c>
+      <c r="AB31" t="s">
+        <v>430</v>
+      </c>
+      <c r="AC31" t="s">
+        <v>430</v>
+      </c>
+      <c r="AD31" t="s">
+        <v>431</v>
+      </c>
+      <c r="AE31" t="s">
+        <v>63</v>
+      </c>
+      <c r="AF31" t="s">
+        <v>356</v>
+      </c>
+      <c r="AG31" t="s">
+        <v>432</v>
+      </c>
+      <c r="AH31" t="s">
+        <v>184</v>
+      </c>
+      <c r="AI31" t="s">
+        <v>341</v>
+      </c>
+      <c r="AJ31" t="s">
+        <v>360</v>
+      </c>
+      <c r="AK31" t="s">
+        <v>433</v>
+      </c>
+      <c r="AL31" t="s">
+        <v>417</v>
+      </c>
+      <c r="AM31" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="32" spans="1:39" x14ac:dyDescent="0.3">
+      <c r="A32" t="s">
+        <v>39</v>
+      </c>
+      <c r="B32" t="s">
+        <v>434</v>
+      </c>
+      <c r="C32" t="s">
+        <v>41</v>
+      </c>
+      <c r="D32" t="s">
+        <v>42</v>
+      </c>
+      <c r="E32" t="s">
+        <v>43</v>
+      </c>
+      <c r="F32" t="s">
+        <v>44</v>
+      </c>
+      <c r="G32" t="s">
+        <v>45</v>
+      </c>
+      <c r="H32" t="s">
+        <v>46</v>
+      </c>
+      <c r="I32" t="s">
+        <v>119</v>
+      </c>
+      <c r="J32" t="s">
+        <v>435</v>
+      </c>
+      <c r="K32" t="s">
+        <v>436</v>
+      </c>
+      <c r="L32" t="s">
         <v>437</v>
       </c>
-      <c r="X31" t="s">
-        <v>425</v>
-      </c>
-      <c r="Y31" t="s">
+      <c r="M32" t="s">
+        <v>51</v>
+      </c>
+      <c r="N32" t="s">
+        <v>52</v>
+      </c>
+      <c r="O32" t="s">
+        <v>220</v>
+      </c>
+      <c r="P32" t="s">
+        <v>44</v>
+      </c>
+      <c r="Q32" t="s">
+        <v>438</v>
+      </c>
+      <c r="R32" t="s">
+        <v>439</v>
+      </c>
+      <c r="S32" t="s">
+        <v>288</v>
+      </c>
+      <c r="T32" t="s">
+        <v>322</v>
+      </c>
+      <c r="U32" t="s">
+        <v>323</v>
+      </c>
+      <c r="V32" t="s">
+        <v>57</v>
+      </c>
+      <c r="W32" t="s">
+        <v>324</v>
+      </c>
+      <c r="X32" t="s">
+        <v>440</v>
+      </c>
+      <c r="Y32" t="s">
         <v>60</v>
       </c>
-      <c r="Z31" t="s">
-        <v>438</v>
-      </c>
-      <c r="AA31" t="s">
-        <v>231</v>
-      </c>
-      <c r="AB31" t="s">
-        <v>439</v>
-      </c>
-      <c r="AC31" t="s">
-        <v>439</v>
-      </c>
-      <c r="AD31" t="s">
-        <v>440</v>
-      </c>
-      <c r="AE31" t="s">
-        <v>44</v>
-      </c>
-      <c r="AF31" t="s">
+      <c r="Z32" t="s">
+        <v>42</v>
+      </c>
+      <c r="AA32" t="s">
+        <v>42</v>
+      </c>
+      <c r="AB32" t="s">
+        <v>324</v>
+      </c>
+      <c r="AC32" t="s">
+        <v>324</v>
+      </c>
+      <c r="AD32" t="s">
+        <v>441</v>
+      </c>
+      <c r="AE32" t="s">
+        <v>63</v>
+      </c>
+      <c r="AF32" t="s">
+        <v>64</v>
+      </c>
+      <c r="AG32" t="s">
+        <v>442</v>
+      </c>
+      <c r="AH32" t="s">
+        <v>443</v>
+      </c>
+      <c r="AI32" t="s">
+        <v>444</v>
+      </c>
+      <c r="AJ32" t="s">
+        <v>360</v>
+      </c>
+      <c r="AK32" t="s">
+        <v>445</v>
+      </c>
+      <c r="AL32" t="s">
+        <v>446</v>
+      </c>
+      <c r="AM32" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="33" spans="1:39" x14ac:dyDescent="0.3">
+      <c r="A33" t="s">
+        <v>39</v>
+      </c>
+      <c r="B33" t="s">
+        <v>447</v>
+      </c>
+      <c r="C33" t="s">
+        <v>41</v>
+      </c>
+      <c r="D33" t="s">
+        <v>448</v>
+      </c>
+      <c r="E33" t="s">
+        <v>44</v>
+      </c>
+      <c r="F33" t="s">
+        <v>44</v>
+      </c>
+      <c r="G33" t="s">
+        <v>44</v>
+      </c>
+      <c r="H33" t="s">
+        <v>329</v>
+      </c>
+      <c r="I33" t="s">
+        <v>203</v>
+      </c>
+      <c r="J33" t="s">
+        <v>449</v>
+      </c>
+      <c r="K33" t="s">
+        <v>450</v>
+      </c>
+      <c r="L33" t="s">
+        <v>451</v>
+      </c>
+      <c r="M33" t="s">
+        <v>51</v>
+      </c>
+      <c r="N33" t="s">
+        <v>52</v>
+      </c>
+      <c r="O33" t="s">
+        <v>53</v>
+      </c>
+      <c r="P33" t="s">
+        <v>452</v>
+      </c>
+      <c r="Q33" t="s">
+        <v>453</v>
+      </c>
+      <c r="R33" t="s">
+        <v>454</v>
+      </c>
+      <c r="S33" t="s">
+        <v>288</v>
+      </c>
+      <c r="T33" t="s">
+        <v>322</v>
+      </c>
+      <c r="U33" t="s">
+        <v>323</v>
+      </c>
+      <c r="V33" t="s">
+        <v>57</v>
+      </c>
+      <c r="W33" t="s">
+        <v>324</v>
+      </c>
+      <c r="X33" t="s">
+        <v>211</v>
+      </c>
+      <c r="Y33" t="s">
+        <v>455</v>
+      </c>
+      <c r="Z33" t="s">
+        <v>42</v>
+      </c>
+      <c r="AA33" t="s">
+        <v>42</v>
+      </c>
+      <c r="AB33" t="s">
+        <v>324</v>
+      </c>
+      <c r="AC33" t="s">
+        <v>324</v>
+      </c>
+      <c r="AD33" t="s">
+        <v>456</v>
+      </c>
+      <c r="AE33" t="s">
+        <v>63</v>
+      </c>
+      <c r="AF33" t="s">
+        <v>64</v>
+      </c>
+      <c r="AG33" t="s">
+        <v>457</v>
+      </c>
+      <c r="AH33" t="s">
+        <v>255</v>
+      </c>
+      <c r="AI33" t="s">
+        <v>256</v>
+      </c>
+      <c r="AJ33" t="s">
+        <v>458</v>
+      </c>
+      <c r="AK33" t="s">
+        <v>459</v>
+      </c>
+      <c r="AL33" t="s">
+        <v>460</v>
+      </c>
+      <c r="AM33" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="34" spans="1:39" x14ac:dyDescent="0.3">
+      <c r="A34" t="s">
+        <v>39</v>
+      </c>
+      <c r="B34" t="s">
+        <v>461</v>
+      </c>
+      <c r="C34" t="s">
+        <v>41</v>
+      </c>
+      <c r="D34" t="s">
+        <v>42</v>
+      </c>
+      <c r="E34" t="s">
+        <v>43</v>
+      </c>
+      <c r="F34" t="s">
+        <v>44</v>
+      </c>
+      <c r="G34" t="s">
+        <v>314</v>
+      </c>
+      <c r="H34" t="s">
+        <v>315</v>
+      </c>
+      <c r="I34" t="s">
+        <v>176</v>
+      </c>
+      <c r="J34" t="s">
+        <v>462</v>
+      </c>
+      <c r="K34" t="s">
+        <v>463</v>
+      </c>
+      <c r="L34" t="s">
+        <v>464</v>
+      </c>
+      <c r="M34" t="s">
+        <v>51</v>
+      </c>
+      <c r="N34" t="s">
+        <v>52</v>
+      </c>
+      <c r="O34" t="s">
+        <v>53</v>
+      </c>
+      <c r="P34" t="s">
+        <v>44</v>
+      </c>
+      <c r="Q34" t="s">
+        <v>465</v>
+      </c>
+      <c r="R34" t="s">
+        <v>466</v>
+      </c>
+      <c r="S34" t="s">
+        <v>288</v>
+      </c>
+      <c r="T34" t="s">
+        <v>322</v>
+      </c>
+      <c r="U34" t="s">
+        <v>323</v>
+      </c>
+      <c r="V34" t="s">
+        <v>57</v>
+      </c>
+      <c r="W34" t="s">
+        <v>307</v>
+      </c>
+      <c r="X34" t="s">
+        <v>384</v>
+      </c>
+      <c r="Y34" t="s">
+        <v>60</v>
+      </c>
+      <c r="Z34" t="s">
+        <v>384</v>
+      </c>
+      <c r="AA34" t="s">
+        <v>184</v>
+      </c>
+      <c r="AB34" t="s">
+        <v>385</v>
+      </c>
+      <c r="AC34" t="s">
+        <v>385</v>
+      </c>
+      <c r="AD34" t="s">
+        <v>310</v>
+      </c>
+      <c r="AE34" t="s">
+        <v>63</v>
+      </c>
+      <c r="AF34" t="s">
+        <v>102</v>
+      </c>
+      <c r="AG34" t="s">
+        <v>467</v>
+      </c>
+      <c r="AH34" t="s">
+        <v>443</v>
+      </c>
+      <c r="AI34" t="s">
+        <v>468</v>
+      </c>
+      <c r="AJ34" t="s">
+        <v>360</v>
+      </c>
+      <c r="AK34" t="s">
+        <v>469</v>
+      </c>
+      <c r="AL34" t="s">
+        <v>460</v>
+      </c>
+      <c r="AM34" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="35" spans="1:39" x14ac:dyDescent="0.3">
+      <c r="A35" t="s">
+        <v>39</v>
+      </c>
+      <c r="B35" t="s">
+        <v>470</v>
+      </c>
+      <c r="C35" t="s">
+        <v>41</v>
+      </c>
+      <c r="D35" t="s">
+        <v>42</v>
+      </c>
+      <c r="E35" t="s">
+        <v>375</v>
+      </c>
+      <c r="F35" t="s">
+        <v>375</v>
+      </c>
+      <c r="G35" t="s">
+        <v>376</v>
+      </c>
+      <c r="H35" t="s">
+        <v>377</v>
+      </c>
+      <c r="I35" t="s">
+        <v>176</v>
+      </c>
+      <c r="J35" t="s">
+        <v>471</v>
+      </c>
+      <c r="K35" t="s">
+        <v>472</v>
+      </c>
+      <c r="L35" t="s">
+        <v>473</v>
+      </c>
+      <c r="M35" t="s">
+        <v>51</v>
+      </c>
+      <c r="N35" t="s">
+        <v>52</v>
+      </c>
+      <c r="O35" t="s">
+        <v>53</v>
+      </c>
+      <c r="P35" t="s">
+        <v>44</v>
+      </c>
+      <c r="Q35" t="s">
+        <v>474</v>
+      </c>
+      <c r="R35" t="s">
+        <v>475</v>
+      </c>
+      <c r="S35" t="s">
+        <v>288</v>
+      </c>
+      <c r="T35" t="s">
+        <v>322</v>
+      </c>
+      <c r="U35" t="s">
+        <v>323</v>
+      </c>
+      <c r="V35" t="s">
+        <v>57</v>
+      </c>
+      <c r="W35" t="s">
+        <v>307</v>
+      </c>
+      <c r="X35" t="s">
+        <v>476</v>
+      </c>
+      <c r="Y35" t="s">
+        <v>477</v>
+      </c>
+      <c r="Z35" t="s">
+        <v>42</v>
+      </c>
+      <c r="AA35" t="s">
+        <v>42</v>
+      </c>
+      <c r="AB35" t="s">
+        <v>307</v>
+      </c>
+      <c r="AC35" t="s">
+        <v>307</v>
+      </c>
+      <c r="AD35" t="s">
+        <v>478</v>
+      </c>
+      <c r="AE35" t="s">
+        <v>63</v>
+      </c>
+      <c r="AF35" t="s">
+        <v>356</v>
+      </c>
+      <c r="AG35" t="s">
+        <v>479</v>
+      </c>
+      <c r="AH35" t="s">
+        <v>340</v>
+      </c>
+      <c r="AI35" t="s">
+        <v>480</v>
+      </c>
+      <c r="AJ35" t="s">
+        <v>360</v>
+      </c>
+      <c r="AK35" t="s">
+        <v>481</v>
+      </c>
+      <c r="AL35" t="s">
+        <v>460</v>
+      </c>
+      <c r="AM35" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="36" spans="1:39" x14ac:dyDescent="0.3">
+      <c r="A36" t="s">
+        <v>39</v>
+      </c>
+      <c r="B36" t="s">
+        <v>482</v>
+      </c>
+      <c r="C36" t="s">
+        <v>41</v>
+      </c>
+      <c r="D36" t="s">
+        <v>211</v>
+      </c>
+      <c r="E36" t="s">
+        <v>483</v>
+      </c>
+      <c r="F36" t="s">
+        <v>420</v>
+      </c>
+      <c r="G36" t="s">
+        <v>484</v>
+      </c>
+      <c r="H36" t="s">
+        <v>484</v>
+      </c>
+      <c r="I36" t="s">
+        <v>44</v>
+      </c>
+      <c r="J36" t="s">
+        <v>485</v>
+      </c>
+      <c r="K36" t="s">
+        <v>486</v>
+      </c>
+      <c r="L36" t="s">
+        <v>487</v>
+      </c>
+      <c r="M36" t="s">
+        <v>51</v>
+      </c>
+      <c r="N36" t="s">
+        <v>52</v>
+      </c>
+      <c r="O36" t="s">
+        <v>488</v>
+      </c>
+      <c r="P36" t="s">
+        <v>44</v>
+      </c>
+      <c r="Q36" t="s">
+        <v>489</v>
+      </c>
+      <c r="R36" t="s">
+        <v>490</v>
+      </c>
+      <c r="S36" t="s">
+        <v>491</v>
+      </c>
+      <c r="T36" t="s">
+        <v>492</v>
+      </c>
+      <c r="U36" t="s">
+        <v>493</v>
+      </c>
+      <c r="V36" t="s">
+        <v>57</v>
+      </c>
+      <c r="W36" t="s">
+        <v>494</v>
+      </c>
+      <c r="X36" t="s">
+        <v>211</v>
+      </c>
+      <c r="Y36" t="s">
+        <v>60</v>
+      </c>
+      <c r="Z36" t="s">
+        <v>495</v>
+      </c>
+      <c r="AA36" t="s">
+        <v>255</v>
+      </c>
+      <c r="AB36" t="s">
+        <v>496</v>
+      </c>
+      <c r="AC36" t="s">
+        <v>496</v>
+      </c>
+      <c r="AD36" t="s">
+        <v>497</v>
+      </c>
+      <c r="AE36" t="s">
+        <v>44</v>
+      </c>
+      <c r="AF36" t="s">
         <v>93</v>
       </c>
-      <c r="AG31" t="s">
-        <v>441</v>
-      </c>
-      <c r="AH31" t="s">
+      <c r="AG36" t="s">
+        <v>498</v>
+      </c>
+      <c r="AH36" t="s">
         <v>189</v>
       </c>
-      <c r="AI31" t="s">
+      <c r="AI36" t="s">
         <v>190</v>
       </c>
-      <c r="AJ31" t="s">
-        <v>334</v>
-      </c>
-      <c r="AK31" t="s">
-        <v>442</v>
-      </c>
-      <c r="AL31" t="s">
-        <v>411</v>
-      </c>
-      <c r="AM31" t="s">
-        <v>443</v>
+      <c r="AJ36" t="s">
+        <v>360</v>
+      </c>
+      <c r="AK36" t="s">
+        <v>499</v>
+      </c>
+      <c r="AL36" t="s">
+        <v>460</v>
+      </c>
+      <c r="AM36" t="s">
+        <v>500</v>
       </c>
     </row>
   </sheetData>

</xml_diff>